<commit_message>
Fix Florence to 2 nights
</commit_message>
<xml_diff>
--- a/europe_nyc_trip_plan.xlsx
+++ b/europe_nyc_trip_plan.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="881" uniqueCount="448">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="711" uniqueCount="443">
   <si>
     <t>Date</t>
   </si>
@@ -553,6 +553,9 @@
     <t>Hotel Davanzati</t>
   </si>
   <si>
+    <t>2</t>
+  </si>
+  <si>
     <t>$240-450</t>
   </si>
   <si>
@@ -868,96 +871,84 @@
     <t>No bag fees</t>
   </si>
   <si>
-    <t>Trains: Ljubljana &gt; Florence (3 legs, 2 ppl)</t>
+    <t>Hotel: Florence (2 nights, 1 room 1 bed)</t>
+  </si>
+  <si>
+    <t>$120</t>
+  </si>
+  <si>
+    <t>$200</t>
+  </si>
+  <si>
+    <t>1 room, 1 double bed x 2 nights</t>
+  </si>
+  <si>
+    <t>Hotel: Rome (1 night, 1 room 1 bed)</t>
+  </si>
+  <si>
+    <t>$60</t>
+  </si>
+  <si>
+    <t>Hotel: Ljubljana (3 nights, 1 room 1 bed)</t>
+  </si>
+  <si>
+    <t>$300</t>
+  </si>
+  <si>
+    <t>1 room, 1 double bed x 3 nights</t>
+  </si>
+  <si>
+    <t>Food: Europe 9 days (2 ppl)</t>
+  </si>
+  <si>
+    <t>$330</t>
+  </si>
+  <si>
+    <t>$570</t>
+  </si>
+  <si>
+    <t>~$35-60/day for 2</t>
+  </si>
+  <si>
+    <t>Sights: Europe 9 days (2 ppl)</t>
+  </si>
+  <si>
+    <t>Colosseum, Uffizi, castle, gorge, Duomo</t>
+  </si>
+  <si>
+    <t>SUBTOTAL: Europe leg</t>
+  </si>
+  <si>
+    <t>$1,674</t>
+  </si>
+  <si>
+    <t>$2,900</t>
+  </si>
+  <si>
+    <t>=== OPTION A: BCN &gt; LA &gt; NYC &gt; Split ===</t>
+  </si>
+  <si>
+    <t>London: food + sights 9 days (2 ppl, free stay)</t>
+  </si>
+  <si>
+    <t>$720</t>
+  </si>
+  <si>
+    <t>$1,260</t>
+  </si>
+  <si>
+    <t>Free stay. Food ~$60-100/day + sights ~$20-40/day for 2</t>
+  </si>
+  <si>
+    <t>Flight: London &gt; Barcelona (2 tix)</t>
+  </si>
+  <si>
+    <t>$50</t>
   </si>
   <si>
     <t>$100</t>
   </si>
   <si>
-    <t>Flight: Florence &gt; London (Vueling, 2 tix)</t>
-  </si>
-  <si>
-    <t>$74</t>
-  </si>
-  <si>
-    <t>$160</t>
-  </si>
-  <si>
-    <t>Cabin bag included</t>
-  </si>
-  <si>
-    <t>Hotel: Rome (1 night, 1 room 1 bed)</t>
-  </si>
-  <si>
-    <t>$60</t>
-  </si>
-  <si>
-    <t>$120</t>
-  </si>
-  <si>
-    <t>Hotel: Ljubljana (3 nights, 1 room 1 bed)</t>
-  </si>
-  <si>
-    <t>$300</t>
-  </si>
-  <si>
-    <t>1 room, 1 double bed x 3 nights</t>
-  </si>
-  <si>
-    <t>Hotel: Florence (3 nights, 1 room 1 bed)</t>
-  </si>
-  <si>
-    <t>$180</t>
-  </si>
-  <si>
-    <t>Food: Europe 9 days (2 ppl)</t>
-  </si>
-  <si>
-    <t>$330</t>
-  </si>
-  <si>
-    <t>$570</t>
-  </si>
-  <si>
-    <t>~$35-60/day for 2</t>
-  </si>
-  <si>
-    <t>Sights: Europe 9 days (2 ppl)</t>
-  </si>
-  <si>
-    <t>Colosseum, Uffizi, castle, gorge, Duomo</t>
-  </si>
-  <si>
-    <t>SUBTOTAL: Europe leg</t>
-  </si>
-  <si>
-    <t>$1,734</t>
-  </si>
-  <si>
-    <t>$3,050</t>
-  </si>
-  <si>
-    <t>=== OPTION A: BCN &gt; LA &gt; NYC &gt; Split ===</t>
-  </si>
-  <si>
-    <t>London: food + sights 9 days (2 ppl, free stay)</t>
-  </si>
-  <si>
-    <t>$720</t>
-  </si>
-  <si>
-    <t>$1,260</t>
-  </si>
-  <si>
-    <t>Free stay. Food ~$60-100/day + sights ~$20-40/day for 2</t>
-  </si>
-  <si>
-    <t>Flight: London &gt; Barcelona (2 tix)</t>
-  </si>
-  <si>
-    <t>$50</t>
-  </si>
-  <si>
     <t>easyJet/Vueling. Cabin bag included</t>
   </si>
   <si>
@@ -970,9 +961,6 @@
     <t>Flight: LAX &gt; NYC (2 tix)</t>
   </si>
   <si>
-    <t>$200</t>
-  </si>
-  <si>
     <t>$500</t>
   </si>
   <si>
@@ -1039,10 +1027,10 @@
     <t>GRAND TOTAL OPTION A</t>
   </si>
   <si>
-    <t>$4,794</t>
-  </si>
-  <si>
-    <t>$8,700</t>
+    <t>$4,734</t>
+  </si>
+  <si>
+    <t>$8,550</t>
   </si>
   <si>
     <t>=== OPTION B: London 22d &gt; NYC &gt; Split ===</t>
@@ -1054,9 +1042,6 @@
     <t>$1,760</t>
   </si>
   <si>
-    <t>$2,900</t>
-  </si>
-  <si>
     <t>Free stay. 22 days food + sights</t>
   </si>
   <si>
@@ -1078,10 +1063,10 @@
     <t>GRAND TOTAL OPTION B</t>
   </si>
   <si>
-    <t>$5,784</t>
-  </si>
-  <si>
-    <t>$10,140</t>
+    <t>$5,724</t>
+  </si>
+  <si>
+    <t>$9,990</t>
   </si>
   <si>
     <t>Day</t>
@@ -1177,10 +1162,10 @@
     <t>$170-260</t>
   </si>
   <si>
+    <t>$0 (checkout, no hotel)</t>
+  </si>
+  <si>
     <t>$20-40</t>
-  </si>
-  <si>
-    <t>$140-240</t>
   </si>
   <si>
     <t>Fly Florence &gt; London</t>
@@ -2564,16 +2549,16 @@
         <v>153</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>165</v>
+        <v>178</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>158</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="9">
@@ -2581,13 +2566,13 @@
         <v>24</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>153</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>165</v>
+        <v>178</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>170</v>
@@ -2596,7 +2581,7 @@
         <v>171</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="10">
@@ -2604,56 +2589,56 @@
         <v>24</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>161</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>165</v>
+        <v>178</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D12" s="3" t="s">
         <v>154</v>
@@ -2665,38 +2650,38 @@
         <v>174</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D13" s="3" t="s">
         <v>154</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>153</v>
@@ -2705,82 +2690,82 @@
         <v>154</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>161</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
   </sheetData>
@@ -2807,13 +2792,13 @@
         <v>146</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>3</v>
@@ -2824,16 +2809,16 @@
         <v>9</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="3">
@@ -2841,16 +2826,16 @@
         <v>9</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="4">
@@ -2858,16 +2843,16 @@
         <v>9</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="5">
@@ -2875,16 +2860,16 @@
         <v>18</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="6">
@@ -2892,16 +2877,16 @@
         <v>18</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="7">
@@ -2909,16 +2894,16 @@
         <v>18</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="8">
@@ -2926,16 +2911,16 @@
         <v>18</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="9">
@@ -2943,16 +2928,16 @@
         <v>24</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="10">
@@ -2960,16 +2945,16 @@
         <v>24</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="11">
@@ -2977,118 +2962,118 @@
         <v>24</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
   </sheetData>
@@ -3104,20 +3089,19 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="38.5"/>
-    <col customWidth="1" min="2" max="2" width="5.88"/>
-    <col customWidth="1" min="3" max="3" width="6.75"/>
+    <col customWidth="1" min="2" max="3" width="5.88"/>
     <col customWidth="1" min="4" max="4" width="42.38"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>3</v>
@@ -3125,83 +3109,77 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>273</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>35</v>
+        <v>274</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>285</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="C6" s="3" t="s">
         <v>286</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="D6" s="2" t="s">
         <v>287</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>288</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>289</v>
       </c>
-      <c r="B7" s="3" t="s">
-        <v>290</v>
-      </c>
       <c r="C7" s="3" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>153</v>
@@ -3209,153 +3187,127 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>292</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>281</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>293</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>294</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>295</v>
+        <v>284</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>296</v>
+        <v>285</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>294</v>
+        <v>287</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>305</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>35</v>
+        <v>301</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="s">
-        <v>306</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>35</v>
+        <v>302</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>284</v>
+        <v>309</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>317</v>
+        <v>286</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>51</v>
@@ -3363,310 +3315,247 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>284</v>
+        <v>309</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>317</v>
+        <v>286</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>284</v>
+        <v>309</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>284</v>
+        <v>309</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>337</v>
+        <v>333</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>338</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>35</v>
+        <v>334</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>341</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>35</v>
+        <v>337</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="s">
-        <v>342</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>35</v>
+        <v>338</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="s">
-        <v>343</v>
+        <v>339</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>345</v>
+        <v>301</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>346</v>
+        <v>341</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="s">
-        <v>347</v>
+        <v>342</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>348</v>
+        <v>343</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>284</v>
+        <v>309</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>317</v>
+        <v>286</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>284</v>
+        <v>309</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>284</v>
+        <v>309</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="s">
-        <v>349</v>
+        <v>344</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>350</v>
+        <v>345</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>351</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D39" s="2" t="s">
-        <v>35</v>
+        <v>346</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="s">
-        <v>352</v>
+        <v>347</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>354</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>35</v>
+        <v>349</v>
       </c>
     </row>
   </sheetData>
@@ -3693,80 +3582,42 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>355</v>
+        <v>350</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>356</v>
+        <v>351</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>147</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>357</v>
+        <v>352</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>359</v>
+        <v>354</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>361</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>35</v>
+        <v>356</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>362</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>35</v>
+        <v>357</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>364</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>35</v>
+        <v>359</v>
       </c>
     </row>
     <row r="4">
@@ -3774,25 +3625,25 @@
         <v>4</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="H4" s="2" t="s">
         <v>365</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>366</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>367</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>368</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>190</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>369</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>370</v>
       </c>
     </row>
     <row r="5">
@@ -3803,7 +3654,7 @@
         <v>9</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>155</v>
@@ -3812,13 +3663,10 @@
         <v>162</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>371</v>
+        <v>366</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>372</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>35</v>
+        <v>367</v>
       </c>
     </row>
     <row r="6">
@@ -3829,22 +3677,19 @@
         <v>12</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>373</v>
+        <v>368</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>374</v>
+        <v>369</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>371</v>
+        <v>366</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>375</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>35</v>
+        <v>370</v>
       </c>
     </row>
     <row r="7">
@@ -3852,25 +3697,22 @@
         <v>14</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>376</v>
+        <v>371</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>377</v>
+        <v>372</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>374</v>
+        <v>369</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>371</v>
+        <v>366</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>378</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>35</v>
+        <v>373</v>
       </c>
     </row>
     <row r="8">
@@ -3881,22 +3723,19 @@
         <v>18</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D8" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="F8" s="2" t="s">
         <v>374</v>
       </c>
-      <c r="E8" s="2" t="s">
-        <v>371</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>379</v>
-      </c>
       <c r="G8" s="2" t="s">
-        <v>380</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>35</v>
+        <v>375</v>
       </c>
     </row>
     <row r="9">
@@ -3907,22 +3746,19 @@
         <v>21</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>381</v>
+        <v>376</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>162</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>371</v>
+        <v>366</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>382</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>35</v>
+        <v>377</v>
       </c>
     </row>
     <row r="10">
@@ -3930,10 +3766,10 @@
         <v>23</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>383</v>
+        <v>378</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>162</v>
@@ -3942,13 +3778,10 @@
         <v>162</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>384</v>
+        <v>379</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>385</v>
-      </c>
-      <c r="H10" s="2" t="s">
-        <v>35</v>
+        <v>380</v>
       </c>
     </row>
     <row r="11">
@@ -3959,22 +3792,19 @@
         <v>27</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>162</v>
+        <v>381</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>162</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>386</v>
+        <v>382</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>387</v>
-      </c>
-      <c r="H11" s="2" t="s">
-        <v>35</v>
+        <v>214</v>
       </c>
     </row>
     <row r="12">
@@ -3982,129 +3812,53 @@
         <v>29</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>388</v>
+        <v>383</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>389</v>
+        <v>384</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>390</v>
+        <v>385</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>391</v>
+        <v>386</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>392</v>
+        <v>387</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
+        <v>388</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>392</v>
+      </c>
+      <c r="G13" s="2" t="s">
         <v>393</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>394</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>190</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>395</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>396</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>397</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>398</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="H14" s="2" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="s">
-        <v>399</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="H15" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="G16" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="H16" s="2" t="s">
-        <v>35</v>
+        <v>394</v>
       </c>
     </row>
     <row r="17">
@@ -4115,22 +3869,22 @@
         <v>38</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>374</v>
+        <v>369</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>371</v>
+        <v>366</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>400</v>
+        <v>395</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>401</v>
+        <v>396</v>
       </c>
     </row>
     <row r="18">
@@ -4138,597 +3892,289 @@
         <v>43</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>402</v>
+        <v>397</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>403</v>
+        <v>398</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>404</v>
+        <v>399</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>405</v>
+        <v>400</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>406</v>
+        <v>401</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>47</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>190</v>
-      </c>
-      <c r="H19" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="G20" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="H20" s="2" t="s">
-        <v>35</v>
+        <v>191</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="s">
-        <v>407</v>
+        <v>402</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>50</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>408</v>
+        <v>403</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>409</v>
+        <v>404</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>410</v>
+        <v>405</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="s">
+        <v>406</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="G22" s="2" t="s">
         <v>411</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>412</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>190</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>413</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>414</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>415</v>
-      </c>
-      <c r="G22" s="2" t="s">
-        <v>416</v>
-      </c>
-      <c r="H22" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="G23" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="H23" s="2" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="s">
-        <v>417</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="G24" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="H24" s="2" t="s">
-        <v>35</v>
+        <v>412</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="s">
-        <v>418</v>
+        <v>413</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>419</v>
+        <v>414</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>110</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>420</v>
+        <v>415</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>421</v>
+        <v>416</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>422</v>
+        <v>417</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>410</v>
+        <v>405</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="s">
-        <v>423</v>
+        <v>418</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>424</v>
+        <v>419</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>425</v>
+        <v>420</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>426</v>
+        <v>421</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>426</v>
+        <v>421</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>425</v>
+        <v>420</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>427</v>
+        <v>422</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="s">
-        <v>428</v>
+        <v>423</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>429</v>
+        <v>424</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>110</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>420</v>
+        <v>415</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>430</v>
+        <v>425</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="G27" s="2" t="s">
         <v>110</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F28" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="G28" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="H28" s="2" t="s">
-        <v>35</v>
+        <v>405</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="s">
-        <v>431</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="E29" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F29" s="2" t="s">
-        <v>35</v>
+        <v>426</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>432</v>
+        <v>427</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>433</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="E30" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F30" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="G30" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="H30" s="2" t="s">
-        <v>35</v>
+        <v>428</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="s">
-        <v>434</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="E31" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F31" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="G31" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="H31" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="E32" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F32" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="G32" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="H32" s="2" t="s">
-        <v>35</v>
+        <v>429</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="s">
-        <v>435</v>
+        <v>430</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>436</v>
+        <v>431</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>395</v>
+        <v>390</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>437</v>
+        <v>432</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>438</v>
+        <v>433</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>439</v>
-      </c>
-      <c r="H33" s="2" t="s">
-        <v>35</v>
+        <v>434</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="s">
-        <v>407</v>
+        <v>402</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>440</v>
+        <v>435</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>441</v>
+        <v>436</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>442</v>
+        <v>437</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>443</v>
+        <v>438</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="s">
+        <v>406</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="G35" s="2" t="s">
         <v>411</v>
-      </c>
-      <c r="B35" s="2" t="s">
-        <v>412</v>
-      </c>
-      <c r="C35" s="3" t="s">
-        <v>190</v>
-      </c>
-      <c r="D35" s="2" t="s">
-        <v>413</v>
-      </c>
-      <c r="E35" s="2" t="s">
-        <v>414</v>
-      </c>
-      <c r="F35" s="2" t="s">
-        <v>415</v>
-      </c>
-      <c r="G35" s="2" t="s">
-        <v>416</v>
-      </c>
-      <c r="H35" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="B36" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="E36" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F36" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="G36" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="H36" s="2" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="s">
-        <v>444</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D37" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="E37" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F37" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="G37" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="H37" s="2" t="s">
-        <v>35</v>
+        <v>439</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="s">
-        <v>445</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="E38" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F38" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="G38" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="H38" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D39" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="E39" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F39" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="G39" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="H39" s="2" t="s">
-        <v>35</v>
+        <v>440</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="s">
-        <v>446</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="E40" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F40" s="2" t="s">
-        <v>35</v>
+        <v>441</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>447</v>
+        <v>442</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>433</v>
+        <v>428</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Correct Florence dates: May 26-28, Ljubljana 4 nights
</commit_message>
<xml_diff>
--- a/europe_nyc_trip_plan.xlsx
+++ b/europe_nyc_trip_plan.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="711" uniqueCount="443">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="881" uniqueCount="448">
   <si>
     <t>Date</t>
   </si>
@@ -82,28 +82,28 @@
     <t>May 25 (Mon)</t>
   </si>
   <si>
+    <t>Ljubljana / Slovenia (extra day)</t>
+  </si>
+  <si>
+    <t>Bonus day! Skocjan caves, Triglav NP, or relax in Ljubljana</t>
+  </si>
+  <si>
+    <t>May 26 (Tue)</t>
+  </si>
+  <si>
     <t>Train: Ljubljana &gt; Florence</t>
   </si>
   <si>
-    <t>Ljubljana &gt; Trieste &gt; Venice &gt; Florence. ~7-8h</t>
-  </si>
-  <si>
-    <t>May 26 (Tue)</t>
+    <t>Ljubljana &gt; Trieste &gt; Venice &gt; Florence. ~7-8h. Arrive evening</t>
+  </si>
+  <si>
+    <t>May 27 (Wed)</t>
   </si>
   <si>
     <t>Florence</t>
   </si>
   <si>
-    <t>Uffizi (BOOK NOW), Ponte Vecchio, Duomo</t>
-  </si>
-  <si>
-    <t>May 27 (Wed)</t>
-  </si>
-  <si>
-    <t>Florence (day 2)</t>
-  </si>
-  <si>
-    <t>Oltrarno, San Lorenzo market, bistecca fiorentina</t>
+    <t>Uffizi (BOOK NOW), Ponte Vecchio, Duomo, bistecca fiorentina</t>
   </si>
   <si>
     <t>May 28 (Thu)</t>
@@ -502,7 +502,7 @@
     <t>Airbnb Trastevere</t>
   </si>
   <si>
-    <t>1 room, 1 bed (Airbnb)</t>
+    <t>1 room, 1 bed</t>
   </si>
   <si>
     <t>$60-100</t>
@@ -514,13 +514,13 @@
     <t>Vander Urbani Resort</t>
   </si>
   <si>
-    <t>3</t>
+    <t>4</t>
   </si>
   <si>
     <t>$90-130</t>
   </si>
   <si>
-    <t>$270-390</t>
+    <t>$360-520</t>
   </si>
   <si>
     <t>Boutique on the river. Best option</t>
@@ -532,7 +532,7 @@
     <t>$70-100</t>
   </si>
   <si>
-    <t>$210-300</t>
+    <t>$280-400</t>
   </si>
   <si>
     <t>Modern, great breakfast</t>
@@ -544,7 +544,7 @@
     <t>$50-80</t>
   </si>
   <si>
-    <t>$150-240</t>
+    <t>$200-320</t>
   </si>
   <si>
     <t>Best value</t>
@@ -556,7 +556,7 @@
     <t>2</t>
   </si>
   <si>
-    <t>$240-450</t>
+    <t>$160-300</t>
   </si>
   <si>
     <t>Central, historic building</t>
@@ -565,6 +565,9 @@
     <t>Hotel Perseo</t>
   </si>
   <si>
+    <t>$140-200</t>
+  </si>
+  <si>
     <t>Near San Lorenzo market</t>
   </si>
   <si>
@@ -574,7 +577,7 @@
     <t>$60-90</t>
   </si>
   <si>
-    <t>$180-270</t>
+    <t>$120-180</t>
   </si>
   <si>
     <t>Artisan neighborhood</t>
@@ -604,9 +607,6 @@
     <t>Generator Barcelona</t>
   </si>
   <si>
-    <t>1 private double room</t>
-  </si>
-  <si>
     <t>Born district. Private double room</t>
   </si>
   <si>
@@ -637,9 +637,6 @@
     <t>7</t>
   </si>
   <si>
-    <t>$120-180</t>
-  </si>
-  <si>
     <t>$840-1,260</t>
   </si>
   <si>
@@ -871,177 +868,198 @@
     <t>No bag fees</t>
   </si>
   <si>
+    <t>Trains: Ljubljana &gt; Florence (3 legs, 2 ppl)</t>
+  </si>
+  <si>
+    <t>$100</t>
+  </si>
+  <si>
+    <t>Flight: Florence &gt; London (Vueling, 2 tix)</t>
+  </si>
+  <si>
+    <t>$74</t>
+  </si>
+  <si>
+    <t>$160</t>
+  </si>
+  <si>
+    <t>Cabin bag included</t>
+  </si>
+  <si>
+    <t>Hotel: Rome (1 night, 1 room 1 bed)</t>
+  </si>
+  <si>
+    <t>$60</t>
+  </si>
+  <si>
+    <t>$120</t>
+  </si>
+  <si>
+    <t>Hotel: Ljubljana (4 nights, 1 room 1 bed)</t>
+  </si>
+  <si>
+    <t>$200</t>
+  </si>
+  <si>
+    <t>$400</t>
+  </si>
+  <si>
+    <t>1 room, 1 double bed x 4 nights (extra Slovenia day!)</t>
+  </si>
+  <si>
     <t>Hotel: Florence (2 nights, 1 room 1 bed)</t>
   </si>
   <si>
-    <t>$120</t>
-  </si>
-  <si>
-    <t>$200</t>
-  </si>
-  <si>
-    <t>1 room, 1 double bed x 2 nights</t>
-  </si>
-  <si>
-    <t>Hotel: Rome (1 night, 1 room 1 bed)</t>
-  </si>
-  <si>
-    <t>$60</t>
-  </si>
-  <si>
-    <t>Hotel: Ljubljana (3 nights, 1 room 1 bed)</t>
+    <t>1 room, 1 double bed x 2 nights (May 26-27)</t>
+  </si>
+  <si>
+    <t>Food: Europe 9 days (2 ppl)</t>
+  </si>
+  <si>
+    <t>$330</t>
+  </si>
+  <si>
+    <t>$570</t>
+  </si>
+  <si>
+    <t>~$35-60/day for 2</t>
+  </si>
+  <si>
+    <t>Sights: Europe 9 days (2 ppl)</t>
   </si>
   <si>
     <t>$300</t>
   </si>
   <si>
-    <t>1 room, 1 double bed x 3 nights</t>
-  </si>
-  <si>
-    <t>Food: Europe 9 days (2 ppl)</t>
-  </si>
-  <si>
-    <t>$330</t>
-  </si>
-  <si>
-    <t>$570</t>
-  </si>
-  <si>
-    <t>~$35-60/day for 2</t>
-  </si>
-  <si>
-    <t>Sights: Europe 9 days (2 ppl)</t>
-  </si>
-  <si>
-    <t>Colosseum, Uffizi, castle, gorge, Duomo</t>
+    <t>Colosseum, Uffizi, castle, gorge, caves</t>
   </si>
   <si>
     <t>SUBTOTAL: Europe leg</t>
   </si>
   <si>
-    <t>$1,674</t>
+    <t>$1,724</t>
+  </si>
+  <si>
+    <t>$3,050</t>
+  </si>
+  <si>
+    <t>=== OPTION A: BCN &gt; LA &gt; NYC &gt; Split ===</t>
+  </si>
+  <si>
+    <t>London: food + sights 9 days (2 ppl, free stay)</t>
+  </si>
+  <si>
+    <t>$720</t>
+  </si>
+  <si>
+    <t>$1,260</t>
+  </si>
+  <si>
+    <t>Free stay. Food ~$60-100/day + sights ~$20-40/day for 2</t>
+  </si>
+  <si>
+    <t>Flight: London &gt; Barcelona (2 tix)</t>
+  </si>
+  <si>
+    <t>$50</t>
+  </si>
+  <si>
+    <t>easyJet/Vueling. Cabin bag included</t>
+  </si>
+  <si>
+    <t>Flight: Barcelona &gt; LAX (LEVEL, 2 tix)</t>
+  </si>
+  <si>
+    <t>LEVEL nonstop. Mon/Wed/Sun only</t>
+  </si>
+  <si>
+    <t>Flight: LAX &gt; NYC (2 tix)</t>
+  </si>
+  <si>
+    <t>$500</t>
+  </si>
+  <si>
+    <t>Hotel: NYC 7 nights (1 room, 1 bed)</t>
+  </si>
+  <si>
+    <t>$840</t>
+  </si>
+  <si>
+    <t>$1,540</t>
+  </si>
+  <si>
+    <t>1 room, 1 bed ($120-220/night). Last shared night Jun 25</t>
+  </si>
+  <si>
+    <t>Food: NYC 7 days (2 ppl)</t>
+  </si>
+  <si>
+    <t>$560</t>
+  </si>
+  <si>
+    <t>~$80-120/day for 2</t>
+  </si>
+  <si>
+    <t>Sights: NYC (2 ppl)</t>
+  </si>
+  <si>
+    <t>Museums, shows, etc.</t>
+  </si>
+  <si>
+    <t>Person A: flight JFK &gt; LAX Jun 26 (1 tix)</t>
+  </si>
+  <si>
+    <t>$250</t>
+  </si>
+  <si>
+    <t>Nonstop JFK&gt;LAX ~5h</t>
+  </si>
+  <si>
+    <t>Person B: Amtrak NYC &gt; Baltimore + Uber (1 person)</t>
+  </si>
+  <si>
+    <t>$110</t>
+  </si>
+  <si>
+    <t>Amtrak $50 + Uber $40-60</t>
+  </si>
+  <si>
+    <t>Person B: flight BWI &gt; LAX Jun 27 (1 tix)</t>
+  </si>
+  <si>
+    <t>Nonstop BWI&gt;LAX ~5h. After wedding Jun 27</t>
+  </si>
+  <si>
+    <t>SUBTOTAL: Option A back half</t>
+  </si>
+  <si>
+    <t>$3,060</t>
+  </si>
+  <si>
+    <t>$5,650</t>
+  </si>
+  <si>
+    <t>GRAND TOTAL OPTION A</t>
+  </si>
+  <si>
+    <t>$4,784</t>
+  </si>
+  <si>
+    <t>$8,700</t>
+  </si>
+  <si>
+    <t>=== OPTION B: London 22d &gt; NYC &gt; Split ===</t>
+  </si>
+  <si>
+    <t>London: food + sights 22 days (2 ppl, free stay)</t>
+  </si>
+  <si>
+    <t>$1,760</t>
   </si>
   <si>
     <t>$2,900</t>
   </si>
   <si>
-    <t>=== OPTION A: BCN &gt; LA &gt; NYC &gt; Split ===</t>
-  </si>
-  <si>
-    <t>London: food + sights 9 days (2 ppl, free stay)</t>
-  </si>
-  <si>
-    <t>$720</t>
-  </si>
-  <si>
-    <t>$1,260</t>
-  </si>
-  <si>
-    <t>Free stay. Food ~$60-100/day + sights ~$20-40/day for 2</t>
-  </si>
-  <si>
-    <t>Flight: London &gt; Barcelona (2 tix)</t>
-  </si>
-  <si>
-    <t>$50</t>
-  </si>
-  <si>
-    <t>$100</t>
-  </si>
-  <si>
-    <t>easyJet/Vueling. Cabin bag included</t>
-  </si>
-  <si>
-    <t>Flight: Barcelona &gt; LAX (LEVEL, 2 tix)</t>
-  </si>
-  <si>
-    <t>LEVEL nonstop. Mon/Wed/Sun only</t>
-  </si>
-  <si>
-    <t>Flight: LAX &gt; NYC (2 tix)</t>
-  </si>
-  <si>
-    <t>$500</t>
-  </si>
-  <si>
-    <t>Hotel: NYC 7 nights (1 room, 1 bed)</t>
-  </si>
-  <si>
-    <t>$840</t>
-  </si>
-  <si>
-    <t>$1,540</t>
-  </si>
-  <si>
-    <t>1 room, 1 bed ($120-220/night). Last shared night Jun 25</t>
-  </si>
-  <si>
-    <t>Food: NYC 7 days (2 ppl)</t>
-  </si>
-  <si>
-    <t>$560</t>
-  </si>
-  <si>
-    <t>~$80-120/day for 2</t>
-  </si>
-  <si>
-    <t>Sights: NYC (2 ppl)</t>
-  </si>
-  <si>
-    <t>Museums, shows, etc.</t>
-  </si>
-  <si>
-    <t>Person A: flight JFK &gt; LAX Jun 26 (1 tix)</t>
-  </si>
-  <si>
-    <t>$250</t>
-  </si>
-  <si>
-    <t>Nonstop JFK&gt;LAX ~5h</t>
-  </si>
-  <si>
-    <t>Person B: Amtrak NYC &gt; Baltimore + Uber (1 person)</t>
-  </si>
-  <si>
-    <t>$110</t>
-  </si>
-  <si>
-    <t>Amtrak $50 + Uber $40-60</t>
-  </si>
-  <si>
-    <t>Person B: flight BWI &gt; LAX Jun 27 (1 tix)</t>
-  </si>
-  <si>
-    <t>Nonstop BWI&gt;LAX ~5h. After wedding Jun 27</t>
-  </si>
-  <si>
-    <t>SUBTOTAL: Option A back half</t>
-  </si>
-  <si>
-    <t>$3,060</t>
-  </si>
-  <si>
-    <t>$5,650</t>
-  </si>
-  <si>
-    <t>GRAND TOTAL OPTION A</t>
-  </si>
-  <si>
-    <t>$4,734</t>
-  </si>
-  <si>
-    <t>$8,550</t>
-  </si>
-  <si>
-    <t>=== OPTION B: London 22d &gt; NYC &gt; Split ===</t>
-  </si>
-  <si>
-    <t>London: food + sights 22 days (2 ppl, free stay)</t>
-  </si>
-  <si>
-    <t>$1,760</t>
-  </si>
-  <si>
     <t>Free stay. 22 days food + sights</t>
   </si>
   <si>
@@ -1063,10 +1081,10 @@
     <t>GRAND TOTAL OPTION B</t>
   </si>
   <si>
-    <t>$5,724</t>
-  </si>
-  <si>
-    <t>$9,990</t>
+    <t>$5,774</t>
+  </si>
+  <si>
+    <t>$10,140</t>
   </si>
   <si>
     <t>Day</t>
@@ -1147,27 +1165,24 @@
     <t>$110-210</t>
   </si>
   <si>
+    <t>$20-40</t>
+  </si>
+  <si>
+    <t>$110-200</t>
+  </si>
+  <si>
     <t>$100-150</t>
   </si>
   <si>
     <t>$200-310</t>
   </si>
   <si>
-    <t>Florence (day 1)</t>
-  </si>
-  <si>
     <t>$50-60</t>
   </si>
   <si>
     <t>$170-260</t>
   </si>
   <si>
-    <t>$0 (checkout, no hotel)</t>
-  </si>
-  <si>
-    <t>$20-40</t>
-  </si>
-  <si>
     <t>Fly Florence &gt; London</t>
   </si>
   <si>
@@ -1186,7 +1201,7 @@
     <t>May 28 - Jun 6 (9d)</t>
   </si>
   <si>
-    <t>London (free, 1 room 1 bed at your place)</t>
+    <t>London (free, 1 room 1 bed)</t>
   </si>
   <si>
     <t>$0 (free)</t>
@@ -1300,7 +1315,7 @@
     <t>OPTION A TOTAL</t>
   </si>
   <si>
-    <t>$4,763-7,853</t>
+    <t>$4,833-7,913</t>
   </si>
   <si>
     <t>NO EXTRA BAGGAGE FEES</t>
@@ -1345,7 +1360,7 @@
     <t>OPTION B TOTAL</t>
   </si>
   <si>
-    <t>$5,023-8,173</t>
+    <t>$5,093-8,233</t>
   </si>
 </sst>
 </file>
@@ -1644,7 +1659,7 @@
     <col customWidth="1" min="1" max="1" width="14.38"/>
     <col customWidth="1" min="2" max="2" width="28.5"/>
     <col customWidth="1" min="3" max="3" width="7.5"/>
-    <col customWidth="1" min="4" max="4" width="43.38"/>
+    <col customWidth="1" min="4" max="4" width="45.88"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2370,7 +2385,7 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="8.13"/>
     <col customWidth="1" min="2" max="2" width="18.75"/>
-    <col customWidth="1" min="3" max="3" width="17.0"/>
+    <col customWidth="1" min="3" max="3" width="16.13"/>
     <col customWidth="1" min="4" max="4" width="16.25"/>
     <col customWidth="1" min="5" max="5" width="12.63"/>
     <col customWidth="1" min="6" max="6" width="10.25"/>
@@ -2540,7 +2555,7 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>177</v>
@@ -2563,7 +2578,7 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>181</v>
@@ -2578,18 +2593,18 @@
         <v>170</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>171</v>
+        <v>182</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>161</v>
@@ -2598,47 +2613,47 @@
         <v>178</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>195</v>
+        <v>153</v>
       </c>
       <c r="D12" s="3" t="s">
         <v>154</v>
@@ -2655,22 +2670,22 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>197</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>195</v>
+        <v>153</v>
       </c>
       <c r="D13" s="3" t="s">
         <v>154</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>198</v>
@@ -2678,7 +2693,7 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>199</v>
@@ -2713,13 +2728,13 @@
         <v>205</v>
       </c>
       <c r="E15" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="F15" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="F15" s="2" t="s">
+      <c r="G15" s="2" t="s">
         <v>207</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="16">
@@ -2727,7 +2742,7 @@
         <v>202</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>204</v>
@@ -2736,13 +2751,13 @@
         <v>205</v>
       </c>
       <c r="E16" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="F16" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="F16" s="2" t="s">
+      <c r="G16" s="2" t="s">
         <v>211</v>
-      </c>
-      <c r="G16" s="2" t="s">
-        <v>212</v>
       </c>
     </row>
     <row r="17">
@@ -2750,7 +2765,7 @@
         <v>202</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>161</v>
@@ -2759,13 +2774,13 @@
         <v>205</v>
       </c>
       <c r="E17" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="F17" s="2" t="s">
         <v>214</v>
       </c>
-      <c r="F17" s="2" t="s">
+      <c r="G17" s="2" t="s">
         <v>215</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>216</v>
       </c>
     </row>
   </sheetData>
@@ -2792,13 +2807,13 @@
         <v>146</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>218</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>219</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>3</v>
@@ -2809,16 +2824,16 @@
         <v>9</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>220</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>222</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="3">
@@ -2826,16 +2841,16 @@
         <v>9</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>224</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>225</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>222</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>226</v>
       </c>
     </row>
     <row r="4">
@@ -2843,16 +2858,16 @@
         <v>9</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>227</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>229</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>230</v>
       </c>
     </row>
     <row r="5">
@@ -2860,16 +2875,16 @@
         <v>18</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>231</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>232</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>222</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>233</v>
       </c>
     </row>
     <row r="6">
@@ -2877,16 +2892,16 @@
         <v>18</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" s="2" t="s">
         <v>235</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>236</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="7">
@@ -2894,16 +2909,16 @@
         <v>18</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>238</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="D7" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>239</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>240</v>
       </c>
     </row>
     <row r="8">
@@ -2911,101 +2926,101 @@
         <v>18</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="D8" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>242</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>222</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>243</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="D9" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>245</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>222</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>246</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="D10" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>248</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>249</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B11" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>250</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="D11" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="E11" s="2" t="s">
         <v>251</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>222</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B12" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="D12" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="E12" s="2" t="s">
         <v>254</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>222</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>255</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B13" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="D13" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="E13" s="2" t="s">
         <v>257</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>258</v>
       </c>
     </row>
     <row r="14">
@@ -3013,16 +3028,16 @@
         <v>202</v>
       </c>
       <c r="B14" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>259</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="D14" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="E14" s="2" t="s">
         <v>260</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>261</v>
       </c>
     </row>
     <row r="15">
@@ -3030,16 +3045,16 @@
         <v>202</v>
       </c>
       <c r="B15" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>262</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="D15" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="E15" s="2" t="s">
         <v>263</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="16">
@@ -3047,16 +3062,16 @@
         <v>202</v>
       </c>
       <c r="B16" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>265</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="D16" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="E16" s="2" t="s">
         <v>266</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>236</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>267</v>
       </c>
     </row>
     <row r="17">
@@ -3064,16 +3079,16 @@
         <v>202</v>
       </c>
       <c r="B17" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>268</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="D17" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="E17" s="2" t="s">
         <v>269</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>222</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>270</v>
       </c>
     </row>
   </sheetData>
@@ -3089,19 +3104,20 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="38.5"/>
-    <col customWidth="1" min="2" max="3" width="5.88"/>
+    <col customWidth="1" min="2" max="2" width="5.88"/>
+    <col customWidth="1" min="3" max="3" width="6.75"/>
     <col customWidth="1" min="4" max="4" width="42.38"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>271</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>272</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>273</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>3</v>
@@ -3109,77 +3125,83 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>274</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>275</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>277</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="2" t="s">
         <v>278</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>279</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>280</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>281</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="2" t="s">
         <v>282</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>283</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>284</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>285</v>
-      </c>
       <c r="C5" s="3" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>285</v>
+        <v>291</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>153</v>
@@ -3187,127 +3209,153 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>282</v>
+        <v>293</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>284</v>
+        <v>296</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>285</v>
+        <v>291</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>286</v>
+        <v>293</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>287</v>
+        <v>297</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>291</v>
+        <v>303</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>298</v>
+        <v>304</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>299</v>
+        <v>305</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>300</v>
+        <v>306</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>301</v>
+        <v>307</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="s">
-        <v>302</v>
+        <v>308</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>303</v>
+        <v>309</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>307</v>
+        <v>313</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>309</v>
+        <v>284</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>291</v>
+        <v>303</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>286</v>
+        <v>293</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>51</v>
@@ -3315,247 +3363,310 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>315</v>
+        <v>320</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>316</v>
+        <v>321</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>316</v>
+        <v>321</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>321</v>
+        <v>326</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>309</v>
+        <v>284</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>286</v>
+        <v>293</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>309</v>
+        <v>284</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="s">
-        <v>327</v>
+        <v>332</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>284</v>
+      </c>
+      <c r="C24" s="3" t="s">
         <v>330</v>
       </c>
-      <c r="B24" s="3" t="s">
-        <v>309</v>
-      </c>
-      <c r="C24" s="3" t="s">
-        <v>325</v>
-      </c>
       <c r="D24" s="2" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>334</v>
+        <v>339</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="s">
-        <v>335</v>
+        <v>340</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>336</v>
+        <v>341</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>337</v>
+        <v>342</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="s">
-        <v>338</v>
+        <v>343</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>301</v>
+        <v>346</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>341</v>
+        <v>347</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="s">
-        <v>342</v>
+        <v>348</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>343</v>
+        <v>349</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="s">
-        <v>315</v>
+        <v>320</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>316</v>
+        <v>321</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>316</v>
+        <v>321</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>321</v>
+        <v>326</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>309</v>
+        <v>284</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>286</v>
+        <v>293</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>309</v>
+        <v>284</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="s">
-        <v>327</v>
+        <v>332</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>284</v>
+      </c>
+      <c r="C37" s="3" t="s">
         <v>330</v>
       </c>
-      <c r="B37" s="3" t="s">
-        <v>309</v>
-      </c>
-      <c r="C37" s="3" t="s">
-        <v>325</v>
-      </c>
       <c r="D37" s="2" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="s">
-        <v>344</v>
+        <v>350</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>345</v>
+        <v>351</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>346</v>
+        <v>352</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="s">
-        <v>347</v>
+        <v>353</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>348</v>
+        <v>354</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>349</v>
+        <v>355</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -3571,7 +3682,7 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="33.25"/>
-    <col customWidth="1" min="2" max="2" width="30.63"/>
+    <col customWidth="1" min="2" max="2" width="28.5"/>
     <col customWidth="1" min="3" max="3" width="11.25"/>
     <col customWidth="1" min="4" max="4" width="29.25"/>
     <col customWidth="1" min="5" max="5" width="15.88"/>
@@ -3582,42 +3693,80 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>350</v>
+        <v>356</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>351</v>
+        <v>357</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>147</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>352</v>
+        <v>358</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>353</v>
+        <v>359</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>354</v>
+        <v>360</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>355</v>
+        <v>361</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>356</v>
+        <v>362</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>357</v>
+        <v>363</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>358</v>
+        <v>364</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>359</v>
+        <v>365</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="4">
@@ -3625,25 +3774,25 @@
         <v>4</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>360</v>
+        <v>366</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>361</v>
+        <v>367</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>362</v>
+        <v>368</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>363</v>
+        <v>369</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>365</v>
+        <v>371</v>
       </c>
     </row>
     <row r="5">
@@ -3654,7 +3803,7 @@
         <v>9</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>155</v>
@@ -3663,10 +3812,13 @@
         <v>162</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>366</v>
+        <v>372</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>367</v>
+        <v>373</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="6">
@@ -3677,19 +3829,22 @@
         <v>12</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>368</v>
+        <v>374</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>366</v>
+        <v>372</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>370</v>
+        <v>376</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="7">
@@ -3697,22 +3852,25 @@
         <v>14</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>371</v>
+        <v>377</v>
       </c>
       <c r="C7" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>372</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="F7" s="2" t="s">
         <v>369</v>
       </c>
-      <c r="E7" s="2" t="s">
-        <v>366</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>363</v>
-      </c>
       <c r="G7" s="2" t="s">
-        <v>373</v>
+        <v>379</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="8">
@@ -3723,19 +3881,22 @@
         <v>18</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>366</v>
+        <v>372</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>375</v>
+        <v>381</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="9">
@@ -3745,20 +3906,23 @@
       <c r="B9" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>376</v>
+      <c r="C9" s="3" t="s">
+        <v>192</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>162</v>
+        <v>375</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>366</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>191</v>
+        <v>372</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>382</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>377</v>
+        <v>383</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="10">
@@ -3766,22 +3930,25 @@
         <v>23</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>378</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>191</v>
+        <v>24</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>384</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>162</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>379</v>
+        <v>372</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>192</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>380</v>
+        <v>385</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="11">
@@ -3792,19 +3959,22 @@
         <v>27</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>381</v>
+        <v>162</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>162</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>382</v>
+        <v>386</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>214</v>
+        <v>387</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="12">
@@ -3812,53 +3982,129 @@
         <v>29</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>383</v>
+        <v>388</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>385</v>
+        <v>390</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>386</v>
+        <v>391</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>387</v>
+        <v>392</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>388</v>
+        <v>393</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>390</v>
+        <v>395</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>391</v>
+        <v>396</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>392</v>
+        <v>397</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>393</v>
+        <v>398</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="s">
-        <v>394</v>
+        <v>399</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="17">
@@ -3869,22 +4115,22 @@
         <v>38</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>366</v>
+        <v>372</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>395</v>
+        <v>400</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>396</v>
+        <v>401</v>
       </c>
     </row>
     <row r="18">
@@ -3892,289 +4138,597 @@
         <v>43</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>397</v>
+        <v>402</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>398</v>
+        <v>403</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>363</v>
+        <v>369</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>399</v>
+        <v>404</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>400</v>
+        <v>405</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>401</v>
+        <v>406</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>47</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="s">
-        <v>402</v>
+        <v>407</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>50</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>403</v>
+        <v>408</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>363</v>
+        <v>369</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>404</v>
+        <v>409</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>405</v>
+        <v>410</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="s">
-        <v>406</v>
+        <v>411</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>407</v>
+        <v>412</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>408</v>
+        <v>413</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>409</v>
+        <v>414</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>410</v>
+        <v>415</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>411</v>
+        <v>416</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="s">
-        <v>412</v>
+        <v>417</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="s">
-        <v>413</v>
+        <v>418</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>414</v>
+        <v>419</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>110</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>415</v>
+        <v>420</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>416</v>
+        <v>421</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>417</v>
+        <v>422</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>405</v>
+        <v>410</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="s">
-        <v>418</v>
+        <v>423</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>419</v>
+        <v>424</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>420</v>
+        <v>425</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>421</v>
+        <v>426</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>421</v>
+        <v>426</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>420</v>
+        <v>425</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>422</v>
+        <v>427</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="s">
-        <v>423</v>
+        <v>428</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>424</v>
+        <v>429</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>110</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>415</v>
+        <v>420</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>425</v>
+        <v>430</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="G27" s="2" t="s">
         <v>110</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>405</v>
+        <v>410</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H28" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="s">
-        <v>426</v>
+        <v>431</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>427</v>
+        <v>432</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>428</v>
+        <v>433</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="s">
-        <v>429</v>
+        <v>434</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H31" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H32" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="s">
-        <v>430</v>
+        <v>435</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>431</v>
+        <v>436</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>390</v>
+        <v>395</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>432</v>
+        <v>437</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>433</v>
+        <v>438</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>434</v>
+        <v>439</v>
+      </c>
+      <c r="H33" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="s">
-        <v>402</v>
+        <v>407</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>435</v>
+        <v>440</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>436</v>
+        <v>441</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>363</v>
+        <v>369</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>437</v>
+        <v>442</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>438</v>
+        <v>443</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="s">
-        <v>406</v>
+        <v>411</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>407</v>
+        <v>412</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>408</v>
+        <v>413</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>409</v>
+        <v>414</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>410</v>
+        <v>415</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>411</v>
+        <v>416</v>
+      </c>
+      <c r="H35" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H36" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="s">
-        <v>439</v>
+        <v>444</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H37" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="s">
-        <v>440</v>
+        <v>445</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H38" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H39" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="s">
-        <v>441</v>
+        <v>446</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>442</v>
+        <v>447</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>428</v>
+        <v>433</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Shift departure to May 22, Ljubljana 2 nights
</commit_message>
<xml_diff>
--- a/europe_nyc_trip_plan.xlsx
+++ b/europe_nyc_trip_plan.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="881" uniqueCount="448">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="857" uniqueCount="439">
   <si>
     <t>Date</t>
   </si>
@@ -31,7 +31,7 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>May 20 (Wed)</t>
+    <t>May 22 (Fri)</t>
   </si>
   <si>
     <t>LAX &gt; Rome</t>
@@ -40,10 +40,10 @@
     <t>Both</t>
   </si>
   <si>
-    <t>ITA Airways AZ621 nonstop. 1 carry-on each</t>
-  </si>
-  <si>
-    <t>May 21 (Thu)</t>
+    <t>ITA Airways AZ621 nonstop ~3:15 PM. Arrive May 23 ~11:55 AM. 1 carry-on each</t>
+  </si>
+  <si>
+    <t>May 23 (Sat)</t>
   </si>
   <si>
     <t>Rome</t>
@@ -52,475 +52,460 @@
     <t>Trastevere, Colosseum, Forum</t>
   </si>
   <si>
-    <t>May 22 (Fri)</t>
+    <t>May 24 (Sun)</t>
   </si>
   <si>
     <t>Train: Rome &gt; Ljubljana</t>
   </si>
   <si>
-    <t>Rome &gt; Venice &gt; Trieste &gt; Ljubljana. ~8-9h</t>
-  </si>
-  <si>
-    <t>May 23 (Sat)</t>
-  </si>
-  <si>
-    <t>Slovenia (Lake Bled)</t>
-  </si>
-  <si>
-    <t>Lake Bled + Vintgar Gorge. Bus from Ljubljana ~1.5h</t>
-  </si>
-  <si>
-    <t>May 24 (Sun)</t>
+    <t>Rome &gt; Venice &gt; Trieste &gt; Ljubljana. ~8-9h. Arrive evening</t>
+  </si>
+  <si>
+    <t>May 25 (Mon)</t>
+  </si>
+  <si>
+    <t>Slovenia (Lake Bled + Vintgar Gorge)</t>
+  </si>
+  <si>
+    <t>Full day: Lake Bled + Vintgar Gorge. Bus from Ljubljana ~1.5h</t>
+  </si>
+  <si>
+    <t>May 26 (Tue)</t>
+  </si>
+  <si>
+    <t>Train: Ljubljana &gt; Florence</t>
+  </si>
+  <si>
+    <t>Ljubljana &gt; Trieste &gt; Venice &gt; Florence. ~7-8h. Arrive evening</t>
+  </si>
+  <si>
+    <t>May 27 (Wed)</t>
+  </si>
+  <si>
+    <t>Florence</t>
+  </si>
+  <si>
+    <t>Uffizi (BOOK NOW), Ponte Vecchio, Duomo, bistecca fiorentina</t>
+  </si>
+  <si>
+    <t>May 28 (Thu)</t>
+  </si>
+  <si>
+    <t>Fly FLR &gt; LGW</t>
+  </si>
+  <si>
+    <t>Vueling ~12:20 PM. Cabin bag included</t>
+  </si>
+  <si>
+    <t>May 28 - Jun 6</t>
+  </si>
+  <si>
+    <t>London (9 days)</t>
+  </si>
+  <si>
+    <t>Free accommodation (1 room, 1 bed)</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>=== OPTION A ===</t>
+  </si>
+  <si>
+    <t>Jun 7 (Sun)</t>
+  </si>
+  <si>
+    <t>Fly LGW &gt; BCN</t>
+  </si>
+  <si>
+    <t>easyJet/Vueling evening. Cabin bag included</t>
+  </si>
+  <si>
+    <t>Jun 7 night</t>
+  </si>
+  <si>
+    <t>Barcelona overnight</t>
+  </si>
+  <si>
+    <t>Born district, tapas, Barceloneta</t>
+  </si>
+  <si>
+    <t>Jun 8 (Mon)</t>
+  </si>
+  <si>
+    <t>Fly BCN &gt; LAX (LEVEL nonstop)</t>
+  </si>
+  <si>
+    <t>LEVEL LL2623 ~2:05 PM. 13h nonstop. Cabin bag included</t>
+  </si>
+  <si>
+    <t>Jun 8 - Jun 18</t>
+  </si>
+  <si>
+    <t>Home in LA</t>
+  </si>
+  <si>
+    <t>Rest, laundry, recharge</t>
+  </si>
+  <si>
+    <t>Jun 18/19</t>
+  </si>
+  <si>
+    <t>Fly LAX &gt; NYC</t>
+  </si>
+  <si>
+    <t>Nonstop ~5h</t>
+  </si>
+  <si>
+    <t>Jun 19 - 25</t>
+  </si>
+  <si>
+    <t>NYC together</t>
+  </si>
+  <si>
+    <t>1 room, 1 bed. Last shared night = Jun 25</t>
+  </si>
+  <si>
+    <t>Jun 26 (Thu)</t>
+  </si>
+  <si>
+    <t>Person A: fly JFK &gt; LAX</t>
+  </si>
+  <si>
+    <t>Person A</t>
+  </si>
+  <si>
+    <t>Nonstop JFK &gt; LAX. ~5h. $100-250</t>
+  </si>
+  <si>
+    <t>Person B: travel to Taneytown</t>
+  </si>
+  <si>
+    <t>Person B</t>
+  </si>
+  <si>
+    <t>Amtrak NYC&gt;Baltimore (~2.5h, $50) + Uber (~1h, $40-60)</t>
+  </si>
+  <si>
+    <t>Jun 27 (Fri)</t>
+  </si>
+  <si>
+    <t>Person B: Wedding, then fly BWI &gt; LAX</t>
+  </si>
+  <si>
+    <t>Wedding. Then BWI &gt; LAX nonstop. ~5h. $100-250</t>
+  </si>
+  <si>
+    <t>Leg</t>
+  </si>
+  <si>
+    <t>Route</t>
+  </si>
+  <si>
+    <t>Airline</t>
+  </si>
+  <si>
+    <t>Duration</t>
+  </si>
+  <si>
+    <t>Price_Per_Person</t>
+  </si>
+  <si>
+    <t>Booking_Notes</t>
+  </si>
+  <si>
+    <t>1. LAX &gt; Rome</t>
+  </si>
+  <si>
+    <t>LAX &gt; FCO (nonstop)</t>
+  </si>
+  <si>
+    <t>ITA Airways (AZ621)</t>
+  </si>
+  <si>
+    <t>~12h</t>
+  </si>
+  <si>
+    <t>$300-500</t>
+  </si>
+  <si>
+    <t>May 22</t>
+  </si>
+  <si>
+    <t>One-way. Book on ITA Airways website. A330-900neo or A350-900</t>
+  </si>
+  <si>
+    <t>2. Florence &gt; London</t>
+  </si>
+  <si>
+    <t>FLR &gt; LGW (nonstop)</t>
+  </si>
+  <si>
+    <t>Vueling (BA codeshare)</t>
+  </si>
+  <si>
+    <t>~2h 25m</t>
+  </si>
+  <si>
+    <t>$37-80</t>
+  </si>
+  <si>
+    <t>May 27</t>
+  </si>
+  <si>
+    <t>Book on Vueling.com. Cabin bag included. ~12:20 PM departure recommended</t>
+  </si>
+  <si>
+    <t>3a. London &gt; Barcelona (Option A)</t>
+  </si>
+  <si>
+    <t>LGW &gt; BCN (nonstop)</t>
+  </si>
+  <si>
+    <t>easyJet or Vueling</t>
+  </si>
+  <si>
+    <t>~2h</t>
+  </si>
+  <si>
+    <t>$25-50</t>
+  </si>
+  <si>
+    <t>Jun 7</t>
+  </si>
+  <si>
+    <t>Book on easyJet.com or Vueling.com. Evening flight</t>
+  </si>
+  <si>
+    <t>3b. Barcelona &gt; LAX (Option A)</t>
+  </si>
+  <si>
+    <t>BCN &gt; LAX (nonstop)</t>
+  </si>
+  <si>
+    <t>LEVEL (LL 2623)</t>
+  </si>
+  <si>
+    <t>~13h</t>
+  </si>
+  <si>
+    <t>$150-300</t>
+  </si>
+  <si>
+    <t>Jun 8</t>
+  </si>
+  <si>
+    <t>LEVEL flies Mon/Wed/Sun ONLY. Book on flylevel.com. Cabin bag included</t>
+  </si>
+  <si>
+    <t>3alt. London &gt; NYC (Option B)</t>
+  </si>
+  <si>
+    <t>LGW &gt; KEF &gt; JFK or LHR &gt; JFK</t>
+  </si>
+  <si>
+    <t>Icelandair / BA / Virgin / JetBlue</t>
+  </si>
+  <si>
+    <t>8-12h</t>
+  </si>
+  <si>
+    <t>$250-500</t>
+  </si>
+  <si>
+    <t>Jun 19</t>
+  </si>
+  <si>
+    <t>Icelandair for budget w/ Iceland stopover option. LHR nonstops pricier but faster</t>
+  </si>
+  <si>
+    <t>4. LAX &gt; NYC (Option A only)</t>
+  </si>
+  <si>
+    <t>LAX &gt; JFK/EWR (nonstop)</t>
+  </si>
+  <si>
+    <t>JetBlue / Delta / Spirit / Southwest</t>
+  </si>
+  <si>
+    <t>~5h</t>
+  </si>
+  <si>
+    <t>$100-250</t>
+  </si>
+  <si>
+    <t>Tons of options. JetBlue Mint is a splurge. Spirit/Frontier cheapest</t>
+  </si>
+  <si>
+    <t>5. BWI &gt; LAX (both options)</t>
+  </si>
+  <si>
+    <t>BWI &gt; LAX (nonstop)</t>
+  </si>
+  <si>
+    <t>Southwest / Spirit / JetBlue</t>
+  </si>
+  <si>
+    <t>Jun 27/28</t>
+  </si>
+  <si>
+    <t>Book closer to date. Southwest has free checked bags if needed</t>
+  </si>
+  <si>
+    <t>Operator</t>
+  </si>
+  <si>
+    <t>Booking</t>
+  </si>
+  <si>
+    <t>Rome &gt; Venice</t>
+  </si>
+  <si>
+    <t>May 24</t>
+  </si>
+  <si>
+    <t>Trenitalia Frecciarossa</t>
+  </si>
+  <si>
+    <t>~3h 40m</t>
+  </si>
+  <si>
+    <t>$20-45 (cheaper if booked early)</t>
+  </si>
+  <si>
+    <t>trenitalia.com - BOOK EARLY for best price</t>
+  </si>
+  <si>
+    <t>Roma Termini &gt; Venezia Santa Lucia. High-speed, reserved seats</t>
+  </si>
+  <si>
+    <t>Venice &gt; Trieste</t>
+  </si>
+  <si>
+    <t>Trenitalia Regional</t>
+  </si>
+  <si>
+    <t>~2h 05m</t>
+  </si>
+  <si>
+    <t>$12-16 (fixed price)</t>
+  </si>
+  <si>
+    <t>Buy at station or trenitalia.com - no reservation needed</t>
+  </si>
+  <si>
+    <t>Venezia S. Lucia &gt; Trieste Centrale. Regional, sit anywhere</t>
+  </si>
+  <si>
+    <t>Trieste &gt; Ljubljana</t>
+  </si>
+  <si>
+    <t>Slovenian Railways (SZ)</t>
+  </si>
+  <si>
+    <t>~2h 50m</t>
+  </si>
+  <si>
+    <t>$11-14 (fixed price)</t>
+  </si>
+  <si>
+    <t>Buy at station - no reservation needed</t>
+  </si>
+  <si>
+    <t>Trieste Centrale &gt; Ljubljana. Cross-border regional</t>
+  </si>
+  <si>
+    <t>Ljubljana &gt; Trieste</t>
+  </si>
+  <si>
+    <t>May 26</t>
+  </si>
+  <si>
+    <t>~2h 40m</t>
+  </si>
+  <si>
+    <t>Ljubljana &gt; Trieste Centrale. Cross-border regional</t>
+  </si>
+  <si>
+    <t>Trieste &gt; Venice</t>
+  </si>
+  <si>
+    <t>Trieste Centrale &gt; Venezia S. Lucia. Regional, sit anywhere</t>
+  </si>
+  <si>
+    <t>Venice &gt; Florence</t>
+  </si>
+  <si>
+    <t>Venezia S. Lucia &gt; Firenze SMN. High-speed, reserved seats</t>
+  </si>
+  <si>
+    <t>City</t>
+  </si>
+  <si>
+    <t>Hotel</t>
+  </si>
+  <si>
+    <t>Room_Type</t>
+  </si>
+  <si>
+    <t>Nights</t>
+  </si>
+  <si>
+    <t>Price_Per_Night</t>
+  </si>
+  <si>
+    <t>Total_Cost</t>
+  </si>
+  <si>
+    <t>Hotel Des Artistes</t>
+  </si>
+  <si>
+    <t>1 room, 1 double bed</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>$60-120</t>
+  </si>
+  <si>
+    <t>Near Termini. Clean, good value</t>
+  </si>
+  <si>
+    <t>Hotel Lancelot</t>
+  </si>
+  <si>
+    <t>$80-150</t>
+  </si>
+  <si>
+    <t>Near Colosseum. Charming</t>
+  </si>
+  <si>
+    <t>Airbnb Trastevere</t>
+  </si>
+  <si>
+    <t>1 room, 1 bed</t>
+  </si>
+  <si>
+    <t>$60-100</t>
+  </si>
+  <si>
+    <t>Best vibe neighborhood</t>
   </si>
   <si>
     <t>Ljubljana</t>
   </si>
   <si>
-    <t>Castle, Central Market. Optional caves</t>
-  </si>
-  <si>
-    <t>May 25 (Mon)</t>
-  </si>
-  <si>
-    <t>Ljubljana / Slovenia (extra day)</t>
-  </si>
-  <si>
-    <t>Bonus day! Skocjan caves, Triglav NP, or relax in Ljubljana</t>
-  </si>
-  <si>
-    <t>May 26 (Tue)</t>
-  </si>
-  <si>
-    <t>Train: Ljubljana &gt; Florence</t>
-  </si>
-  <si>
-    <t>Ljubljana &gt; Trieste &gt; Venice &gt; Florence. ~7-8h. Arrive evening</t>
-  </si>
-  <si>
-    <t>May 27 (Wed)</t>
-  </si>
-  <si>
-    <t>Florence</t>
-  </si>
-  <si>
-    <t>Uffizi (BOOK NOW), Ponte Vecchio, Duomo, bistecca fiorentina</t>
-  </si>
-  <si>
-    <t>May 28 (Thu)</t>
-  </si>
-  <si>
-    <t>Fly FLR &gt; LGW</t>
-  </si>
-  <si>
-    <t>Vueling ~12:20 PM. Cabin bag included</t>
-  </si>
-  <si>
-    <t>May 28 - Jun 6</t>
-  </si>
-  <si>
-    <t>London (9 days)</t>
-  </si>
-  <si>
-    <t>Free accommodation (1 room, 1 bed)</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>=== OPTION A ===</t>
-  </si>
-  <si>
-    <t>Jun 7 (Sun)</t>
-  </si>
-  <si>
-    <t>Fly LGW &gt; BCN</t>
-  </si>
-  <si>
-    <t>easyJet/Vueling evening. Cabin bag included</t>
-  </si>
-  <si>
-    <t>Jun 7 night</t>
-  </si>
-  <si>
-    <t>Barcelona overnight</t>
-  </si>
-  <si>
-    <t>Born district, tapas, Barceloneta</t>
-  </si>
-  <si>
-    <t>Jun 8 (Mon)</t>
-  </si>
-  <si>
-    <t>Fly BCN &gt; LAX (LEVEL nonstop)</t>
-  </si>
-  <si>
-    <t>LEVEL LL2623 ~2:05 PM. 13h nonstop. Cabin bag included</t>
-  </si>
-  <si>
-    <t>Jun 8 - Jun 18</t>
-  </si>
-  <si>
-    <t>Home in LA</t>
-  </si>
-  <si>
-    <t>Rest, laundry, recharge</t>
-  </si>
-  <si>
-    <t>Jun 18/19</t>
-  </si>
-  <si>
-    <t>Fly LAX &gt; NYC</t>
-  </si>
-  <si>
-    <t>Nonstop ~5h</t>
-  </si>
-  <si>
-    <t>Jun 19 - 25</t>
-  </si>
-  <si>
-    <t>NYC together</t>
-  </si>
-  <si>
-    <t>1 room, 1 bed. Last shared night = Jun 25</t>
-  </si>
-  <si>
-    <t>Jun 26 (Thu)</t>
-  </si>
-  <si>
-    <t>Person A: fly JFK &gt; LAX</t>
-  </si>
-  <si>
-    <t>Person A</t>
-  </si>
-  <si>
-    <t>Nonstop JFK &gt; LAX. ~5h. $100-250</t>
-  </si>
-  <si>
-    <t>Person B: travel to Taneytown</t>
-  </si>
-  <si>
-    <t>Person B</t>
-  </si>
-  <si>
-    <t>Amtrak NYC&gt;Baltimore (~2.5h, $50) + Uber (~1h, $40-60)</t>
-  </si>
-  <si>
-    <t>Jun 27 (Fri)</t>
-  </si>
-  <si>
-    <t>Person B: Wedding, then fly BWI &gt; LAX</t>
-  </si>
-  <si>
-    <t>Wedding. Then BWI &gt; LAX nonstop. ~5h. $100-250</t>
-  </si>
-  <si>
-    <t>Leg</t>
-  </si>
-  <si>
-    <t>Route</t>
-  </si>
-  <si>
-    <t>Airline</t>
-  </si>
-  <si>
-    <t>Duration</t>
-  </si>
-  <si>
-    <t>Price_Per_Person</t>
-  </si>
-  <si>
-    <t>Booking_Notes</t>
-  </si>
-  <si>
-    <t>1. LAX &gt; Rome</t>
-  </si>
-  <si>
-    <t>LAX &gt; FCO (nonstop)</t>
-  </si>
-  <si>
-    <t>ITA Airways (AZ621)</t>
-  </si>
-  <si>
-    <t>~12h</t>
-  </si>
-  <si>
-    <t>$300-500</t>
-  </si>
-  <si>
-    <t>May 20</t>
-  </si>
-  <si>
-    <t>One-way. Book on ITA Airways website. A330-900neo or A350-900</t>
-  </si>
-  <si>
-    <t>2. Florence &gt; London</t>
-  </si>
-  <si>
-    <t>FLR &gt; LGW (nonstop)</t>
-  </si>
-  <si>
-    <t>Vueling (BA codeshare)</t>
-  </si>
-  <si>
-    <t>~2h 25m</t>
-  </si>
-  <si>
-    <t>$37-80</t>
-  </si>
-  <si>
-    <t>May 27</t>
-  </si>
-  <si>
-    <t>Book on Vueling.com. Cabin bag included. ~12:20 PM departure recommended</t>
-  </si>
-  <si>
-    <t>3a. London &gt; Barcelona (Option A)</t>
-  </si>
-  <si>
-    <t>LGW &gt; BCN (nonstop)</t>
-  </si>
-  <si>
-    <t>easyJet or Vueling</t>
-  </si>
-  <si>
-    <t>~2h</t>
-  </si>
-  <si>
-    <t>$25-50</t>
-  </si>
-  <si>
-    <t>Jun 7</t>
-  </si>
-  <si>
-    <t>Book on easyJet.com or Vueling.com. Evening flight</t>
-  </si>
-  <si>
-    <t>3b. Barcelona &gt; LAX (Option A)</t>
-  </si>
-  <si>
-    <t>BCN &gt; LAX (nonstop)</t>
-  </si>
-  <si>
-    <t>LEVEL (LL 2623)</t>
-  </si>
-  <si>
-    <t>~13h</t>
-  </si>
-  <si>
-    <t>$150-300</t>
-  </si>
-  <si>
-    <t>Jun 8</t>
-  </si>
-  <si>
-    <t>LEVEL flies Mon/Wed/Sun ONLY. Book on flylevel.com. Cabin bag included</t>
-  </si>
-  <si>
-    <t>3alt. London &gt; NYC (Option B)</t>
-  </si>
-  <si>
-    <t>LGW &gt; KEF &gt; JFK or LHR &gt; JFK</t>
-  </si>
-  <si>
-    <t>Icelandair / BA / Virgin / JetBlue</t>
-  </si>
-  <si>
-    <t>8-12h</t>
-  </si>
-  <si>
-    <t>$250-500</t>
-  </si>
-  <si>
-    <t>Jun 19</t>
-  </si>
-  <si>
-    <t>Icelandair for budget w/ Iceland stopover option. LHR nonstops pricier but faster</t>
-  </si>
-  <si>
-    <t>4. LAX &gt; NYC (Option A only)</t>
-  </si>
-  <si>
-    <t>LAX &gt; JFK/EWR (nonstop)</t>
-  </si>
-  <si>
-    <t>JetBlue / Delta / Spirit / Southwest</t>
-  </si>
-  <si>
-    <t>~5h</t>
-  </si>
-  <si>
-    <t>$100-250</t>
-  </si>
-  <si>
-    <t>Tons of options. JetBlue Mint is a splurge. Spirit/Frontier cheapest</t>
-  </si>
-  <si>
-    <t>5. BWI &gt; LAX (both options)</t>
-  </si>
-  <si>
-    <t>BWI &gt; LAX (nonstop)</t>
-  </si>
-  <si>
-    <t>Southwest / Spirit / JetBlue</t>
-  </si>
-  <si>
-    <t>Jun 27/28</t>
-  </si>
-  <si>
-    <t>Book closer to date. Southwest has free checked bags if needed</t>
-  </si>
-  <si>
-    <t>Operator</t>
-  </si>
-  <si>
-    <t>Booking</t>
-  </si>
-  <si>
-    <t>Rome &gt; Venice</t>
-  </si>
-  <si>
-    <t>May 22</t>
-  </si>
-  <si>
-    <t>Trenitalia Frecciarossa</t>
-  </si>
-  <si>
-    <t>~3h 40m</t>
-  </si>
-  <si>
-    <t>$20-45 (cheaper if booked early)</t>
-  </si>
-  <si>
-    <t>trenitalia.com - BOOK EARLY for best price</t>
-  </si>
-  <si>
-    <t>Roma Termini &gt; Venezia Santa Lucia. High-speed, reserved seats</t>
-  </si>
-  <si>
-    <t>Venice &gt; Trieste</t>
-  </si>
-  <si>
-    <t>Trenitalia Regional</t>
-  </si>
-  <si>
-    <t>~2h 05m</t>
-  </si>
-  <si>
-    <t>$12-16 (fixed price)</t>
-  </si>
-  <si>
-    <t>Buy at station or trenitalia.com - no reservation needed</t>
-  </si>
-  <si>
-    <t>Venezia S. Lucia &gt; Trieste Centrale. Regional, sit anywhere</t>
-  </si>
-  <si>
-    <t>Trieste &gt; Ljubljana</t>
-  </si>
-  <si>
-    <t>Slovenian Railways (SZ)</t>
-  </si>
-  <si>
-    <t>~2h 50m</t>
-  </si>
-  <si>
-    <t>$11-14 (fixed price)</t>
-  </si>
-  <si>
-    <t>Buy at station - no reservation needed</t>
-  </si>
-  <si>
-    <t>Trieste Centrale &gt; Ljubljana. Cross-border regional</t>
-  </si>
-  <si>
-    <t>Ljubljana &gt; Trieste</t>
-  </si>
-  <si>
-    <t>May 25</t>
-  </si>
-  <si>
-    <t>~2h 40m</t>
-  </si>
-  <si>
-    <t>Ljubljana &gt; Trieste Centrale. Cross-border regional</t>
-  </si>
-  <si>
-    <t>Trieste &gt; Venice</t>
-  </si>
-  <si>
-    <t>Trieste Centrale &gt; Venezia S. Lucia. Regional, sit anywhere</t>
-  </si>
-  <si>
-    <t>Venice &gt; Florence</t>
-  </si>
-  <si>
-    <t>Venezia S. Lucia &gt; Firenze SMN. High-speed, reserved seats</t>
-  </si>
-  <si>
-    <t>City</t>
-  </si>
-  <si>
-    <t>Hotel</t>
-  </si>
-  <si>
-    <t>Room_Type</t>
-  </si>
-  <si>
-    <t>Nights</t>
-  </si>
-  <si>
-    <t>Price_Per_Night</t>
-  </si>
-  <si>
-    <t>Total_Cost</t>
-  </si>
-  <si>
-    <t>Hotel Des Artistes</t>
-  </si>
-  <si>
-    <t>1 room, 1 double bed</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>$60-120</t>
-  </si>
-  <si>
-    <t>Near Termini. Clean, good value</t>
-  </si>
-  <si>
-    <t>Hotel Lancelot</t>
-  </si>
-  <si>
-    <t>$80-150</t>
-  </si>
-  <si>
-    <t>Near Colosseum. Charming</t>
-  </si>
-  <si>
-    <t>Airbnb Trastevere</t>
-  </si>
-  <si>
-    <t>1 room, 1 bed</t>
-  </si>
-  <si>
-    <t>$60-100</t>
-  </si>
-  <si>
-    <t>Best vibe neighborhood</t>
-  </si>
-  <si>
     <t>Vander Urbani Resort</t>
   </si>
   <si>
-    <t>4</t>
+    <t>2</t>
   </si>
   <si>
     <t>$90-130</t>
   </si>
   <si>
-    <t>$360-520</t>
+    <t>$180-260</t>
   </si>
   <si>
     <t>Boutique on the river. Best option</t>
@@ -532,7 +517,7 @@
     <t>$70-100</t>
   </si>
   <si>
-    <t>$280-400</t>
+    <t>$140-200</t>
   </si>
   <si>
     <t>Modern, great breakfast</t>
@@ -544,7 +529,7 @@
     <t>$50-80</t>
   </si>
   <si>
-    <t>$200-320</t>
+    <t>$100-160</t>
   </si>
   <si>
     <t>Best value</t>
@@ -553,9 +538,6 @@
     <t>Hotel Davanzati</t>
   </si>
   <si>
-    <t>2</t>
-  </si>
-  <si>
     <t>$160-300</t>
   </si>
   <si>
@@ -565,9 +547,6 @@
     <t>Hotel Perseo</t>
   </si>
   <si>
-    <t>$140-200</t>
-  </si>
-  <si>
     <t>Near San Lorenzo market</t>
   </si>
   <si>
@@ -853,7 +832,7 @@
     <t>$1,000</t>
   </si>
   <si>
-    <t>Book ASAP</t>
+    <t>Book ASAP. Departs ~3:15 PM May 22</t>
   </si>
   <si>
     <t>Trains: Rome &gt; Ljubljana (3 legs, 2 ppl)</t>
@@ -895,16 +874,16 @@
     <t>$120</t>
   </si>
   <si>
-    <t>Hotel: Ljubljana (4 nights, 1 room 1 bed)</t>
+    <t>1 room, 1 double bed (May 23)</t>
+  </si>
+  <si>
+    <t>Hotel: Ljubljana (2 nights, 1 room 1 bed)</t>
   </si>
   <si>
     <t>$200</t>
   </si>
   <si>
-    <t>$400</t>
-  </si>
-  <si>
-    <t>1 room, 1 double bed x 4 nights (extra Slovenia day!)</t>
+    <t>1 room, 1 double bed x 2 nights (May 24-25)</t>
   </si>
   <si>
     <t>Hotel: Florence (2 nights, 1 room 1 bed)</t>
@@ -913,63 +892,69 @@
     <t>1 room, 1 double bed x 2 nights (May 26-27)</t>
   </si>
   <si>
-    <t>Food: Europe 9 days (2 ppl)</t>
-  </si>
-  <si>
-    <t>$330</t>
-  </si>
-  <si>
-    <t>$570</t>
+    <t>Food: Europe 7 days (2 ppl)</t>
+  </si>
+  <si>
+    <t>$290</t>
+  </si>
+  <si>
+    <t>$490</t>
   </si>
   <si>
     <t>~$35-60/day for 2</t>
   </si>
   <si>
-    <t>Sights: Europe 9 days (2 ppl)</t>
+    <t>Sights: Europe 7 days (2 ppl)</t>
+  </si>
+  <si>
+    <t>$130</t>
+  </si>
+  <si>
+    <t>$260</t>
+  </si>
+  <si>
+    <t>Colosseum, Uffizi, Bled, gorge</t>
+  </si>
+  <si>
+    <t>SUBTOTAL: Europe leg</t>
+  </si>
+  <si>
+    <t>$1,564</t>
+  </si>
+  <si>
+    <t>$2,730</t>
+  </si>
+  <si>
+    <t>=== OPTION A: BCN &gt; LA &gt; NYC &gt; Split ===</t>
+  </si>
+  <si>
+    <t>London: food + sights 9 days (2 ppl, free stay)</t>
+  </si>
+  <si>
+    <t>$720</t>
+  </si>
+  <si>
+    <t>$1,260</t>
+  </si>
+  <si>
+    <t>Free stay. Food ~$60-100/day + sights ~$20-40/day for 2</t>
+  </si>
+  <si>
+    <t>Flight: London &gt; Barcelona (2 tix)</t>
+  </si>
+  <si>
+    <t>$50</t>
+  </si>
+  <si>
+    <t>easyJet/Vueling. Cabin bag included</t>
+  </si>
+  <si>
+    <t>Flight: Barcelona &gt; LAX (LEVEL, 2 tix)</t>
   </si>
   <si>
     <t>$300</t>
   </si>
   <si>
-    <t>Colosseum, Uffizi, castle, gorge, caves</t>
-  </si>
-  <si>
-    <t>SUBTOTAL: Europe leg</t>
-  </si>
-  <si>
-    <t>$1,724</t>
-  </si>
-  <si>
-    <t>$3,050</t>
-  </si>
-  <si>
-    <t>=== OPTION A: BCN &gt; LA &gt; NYC &gt; Split ===</t>
-  </si>
-  <si>
-    <t>London: food + sights 9 days (2 ppl, free stay)</t>
-  </si>
-  <si>
-    <t>$720</t>
-  </si>
-  <si>
-    <t>$1,260</t>
-  </si>
-  <si>
-    <t>Free stay. Food ~$60-100/day + sights ~$20-40/day for 2</t>
-  </si>
-  <si>
-    <t>Flight: London &gt; Barcelona (2 tix)</t>
-  </si>
-  <si>
-    <t>$50</t>
-  </si>
-  <si>
-    <t>easyJet/Vueling. Cabin bag included</t>
-  </si>
-  <si>
-    <t>Flight: Barcelona &gt; LAX (LEVEL, 2 tix)</t>
-  </si>
-  <si>
     <t>LEVEL nonstop. Mon/Wed/Sun only</t>
   </si>
   <si>
@@ -1042,10 +1027,10 @@
     <t>GRAND TOTAL OPTION A</t>
   </si>
   <si>
-    <t>$4,784</t>
-  </si>
-  <si>
-    <t>$8,700</t>
+    <t>$4,624</t>
+  </si>
+  <si>
+    <t>$8,380</t>
   </si>
   <si>
     <t>=== OPTION B: London 22d &gt; NYC &gt; Split ===</t>
@@ -1081,10 +1066,10 @@
     <t>GRAND TOTAL OPTION B</t>
   </si>
   <si>
-    <t>$5,774</t>
-  </si>
-  <si>
-    <t>$10,140</t>
+    <t>$5,614</t>
+  </si>
+  <si>
+    <t>$9,820</t>
   </si>
   <si>
     <t>Day</t>
@@ -1150,7 +1135,7 @@
     <t>$180-310</t>
   </si>
   <si>
-    <t>Lake Bled day trip</t>
+    <t>Lake Bled + Vintgar Gorge</t>
   </si>
   <si>
     <t>$14-28</t>
@@ -1159,18 +1144,6 @@
     <t>$124-218</t>
   </si>
   <si>
-    <t>$20-50</t>
-  </si>
-  <si>
-    <t>$110-210</t>
-  </si>
-  <si>
-    <t>$20-40</t>
-  </si>
-  <si>
-    <t>$110-200</t>
-  </si>
-  <si>
     <t>$100-150</t>
   </si>
   <si>
@@ -1315,7 +1288,7 @@
     <t>OPTION A TOTAL</t>
   </si>
   <si>
-    <t>$4,833-7,913</t>
+    <t>$4,613-7,613</t>
   </si>
   <si>
     <t>NO EXTRA BAGGAGE FEES</t>
@@ -1360,7 +1333,7 @@
     <t>OPTION B TOTAL</t>
   </si>
   <si>
-    <t>$5,093-8,233</t>
+    <t>$4,873-7,933</t>
   </si>
 </sst>
 </file>
@@ -1659,7 +1632,7 @@
     <col customWidth="1" min="1" max="1" width="14.38"/>
     <col customWidth="1" min="2" max="2" width="28.5"/>
     <col customWidth="1" min="3" max="3" width="7.5"/>
-    <col customWidth="1" min="4" max="4" width="45.88"/>
+    <col customWidth="1" min="4" max="4" width="59.5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1793,55 +1766,55 @@
         <v>29</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="s">
-        <v>32</v>
-      </c>
       <c r="B11" s="2" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>6</v>
+        <v>29</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>35</v>
+        <v>6</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="s">
-        <v>36</v>
+      <c r="A13" s="2" t="s">
+        <v>34</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>35</v>
+        <v>6</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14">
@@ -1873,7 +1846,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="3" t="s">
         <v>43</v>
       </c>
       <c r="B16" s="2" t="s">
@@ -1901,87 +1874,59 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="s">
-        <v>49</v>
+      <c r="A18" s="2" t="s">
+        <v>29</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>6</v>
+        <v>29</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>51</v>
+        <v>29</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>52</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="s">
-        <v>35</v>
+        <v>49</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>35</v>
+        <v>53</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>35</v>
+        <v>54</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>35</v>
+        <v>55</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>58</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -2007,186 +1952,186 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>71</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>78</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>85</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="G5" s="2" t="s">
         <v>92</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>99</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="D8" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="F8" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="G8" s="2" t="s">
         <v>110</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>116</v>
       </c>
     </row>
   </sheetData>
@@ -2212,22 +2157,22 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>3</v>
@@ -2235,140 +2180,140 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>119</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="E5" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="G5" s="2" t="s">
         <v>135</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="G7" s="2" t="s">
         <v>139</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>145</v>
       </c>
     </row>
   </sheetData>
@@ -2394,22 +2339,22 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>3</v>
@@ -2420,22 +2365,22 @@
         <v>9</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
     </row>
     <row r="3">
@@ -2443,22 +2388,22 @@
         <v>9</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="C3" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>153</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="4">
@@ -2466,321 +2411,321 @@
         <v>9</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>18</v>
+        <v>158</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>18</v>
+        <v>158</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="D6" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="E6" s="2" t="s">
-        <v>170</v>
-      </c>
       <c r="F6" s="2" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>18</v>
+        <v>158</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>178</v>
+        <v>160</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>178</v>
+        <v>160</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>182</v>
+        <v>166</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="D10" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="E10" s="2" t="s">
-        <v>185</v>
-      </c>
       <c r="F10" s="2" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="G14" s="2" t="s">
         <v>194</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>204</v>
+        <v>197</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="E16" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="C16" s="2" t="s">
+      <c r="F16" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="G16" s="2" t="s">
         <v>204</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>205</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="G16" s="2" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
     </row>
   </sheetData>
@@ -2804,16 +2749,16 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>3</v>
@@ -2824,16 +2769,16 @@
         <v>9</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
     </row>
     <row r="3">
@@ -2841,16 +2786,16 @@
         <v>9</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
     </row>
     <row r="4">
@@ -2858,237 +2803,237 @@
         <v>9</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>18</v>
+        <v>158</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>18</v>
+        <v>158</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>18</v>
+        <v>158</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>18</v>
+        <v>158</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>248</v>
+        <v>241</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>257</v>
+        <v>250</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>258</v>
+        <v>251</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>260</v>
+        <v>253</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>261</v>
+        <v>254</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>262</v>
+        <v>255</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>263</v>
+        <v>256</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>264</v>
+        <v>257</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>265</v>
+        <v>258</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>268</v>
+        <v>261</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
   </sheetData>
@@ -3104,20 +3049,19 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="38.5"/>
-    <col customWidth="1" min="2" max="2" width="5.88"/>
-    <col customWidth="1" min="3" max="3" width="6.75"/>
+    <col customWidth="1" min="2" max="3" width="5.88"/>
     <col customWidth="1" min="4" max="4" width="42.38"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>270</v>
+        <v>263</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>271</v>
+        <v>264</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>272</v>
+        <v>265</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>3</v>
@@ -3125,548 +3069,548 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>273</v>
+        <v>266</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>274</v>
+        <v>267</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>275</v>
+        <v>268</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>278</v>
+        <v>271</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>279</v>
+        <v>272</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>280</v>
+        <v>273</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>281</v>
+        <v>274</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>282</v>
+        <v>275</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>284</v>
+        <v>277</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>281</v>
+        <v>274</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>282</v>
+        <v>275</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>285</v>
+        <v>278</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>286</v>
+        <v>279</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>287</v>
+        <v>280</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>288</v>
+        <v>281</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>289</v>
+        <v>282</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>290</v>
+        <v>283</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>291</v>
+        <v>284</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>153</v>
+        <v>285</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>293</v>
+        <v>277</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>294</v>
+        <v>287</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>295</v>
+        <v>288</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>296</v>
+        <v>289</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>291</v>
+        <v>284</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>293</v>
+        <v>287</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>297</v>
+        <v>290</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>298</v>
+        <v>291</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>299</v>
+        <v>292</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>300</v>
+        <v>293</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>301</v>
+        <v>294</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>302</v>
+        <v>295</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>281</v>
+        <v>296</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>303</v>
+        <v>297</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>306</v>
+        <v>300</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>307</v>
+        <v>301</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="s">
-        <v>308</v>
+        <v>302</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>310</v>
+        <v>304</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>311</v>
+        <v>305</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>312</v>
+        <v>306</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>313</v>
+        <v>307</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>314</v>
+        <v>308</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>284</v>
+        <v>277</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>315</v>
+        <v>309</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>316</v>
+        <v>310</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>303</v>
+        <v>311</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>317</v>
+        <v>312</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="s">
-        <v>318</v>
+        <v>313</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>293</v>
+        <v>287</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>319</v>
+        <v>314</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>320</v>
+        <v>315</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>322</v>
+        <v>317</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>323</v>
+        <v>318</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>325</v>
+        <v>320</v>
       </c>
       <c r="C20" s="3" t="s">
+        <v>316</v>
+      </c>
+      <c r="D20" s="2" t="s">
         <v>321</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>326</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="s">
-        <v>327</v>
+        <v>322</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>284</v>
+        <v>277</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>293</v>
+        <v>287</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>328</v>
+        <v>323</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="s">
-        <v>329</v>
+        <v>324</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>284</v>
+        <v>277</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>331</v>
+        <v>326</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>280</v>
+        <v>273</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>334</v>
+        <v>329</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="s">
-        <v>335</v>
+        <v>330</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>284</v>
+        <v>277</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>336</v>
+        <v>331</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="s">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="s">
-        <v>344</v>
+        <v>339</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>346</v>
+        <v>341</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>347</v>
+        <v>342</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="s">
-        <v>348</v>
+        <v>343</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>319</v>
+        <v>314</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>349</v>
+        <v>344</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="s">
-        <v>320</v>
+        <v>315</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>322</v>
+        <v>317</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>323</v>
+        <v>318</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>325</v>
+        <v>320</v>
       </c>
       <c r="C33" s="3" t="s">
+        <v>316</v>
+      </c>
+      <c r="D33" s="2" t="s">
         <v>321</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>326</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="s">
-        <v>327</v>
+        <v>322</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>284</v>
+        <v>277</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>293</v>
+        <v>287</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>328</v>
+        <v>323</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="s">
-        <v>329</v>
+        <v>324</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>284</v>
+        <v>277</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>331</v>
+        <v>326</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>280</v>
+        <v>273</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>334</v>
+        <v>329</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="s">
-        <v>335</v>
+        <v>330</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>284</v>
+        <v>277</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>336</v>
+        <v>331</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="s">
-        <v>350</v>
+        <v>345</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>351</v>
+        <v>346</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>352</v>
+        <v>347</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>355</v>
+        <v>350</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -3693,80 +3637,80 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>356</v>
+        <v>351</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>357</v>
+        <v>352</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>359</v>
+        <v>354</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>361</v>
+        <v>356</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>362</v>
+        <v>357</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>364</v>
+        <v>359</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>365</v>
+        <v>360</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4">
@@ -3774,25 +3718,25 @@
         <v>4</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="H4" s="2" t="s">
         <v>366</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>367</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>368</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>369</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>370</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>371</v>
       </c>
     </row>
     <row r="5">
@@ -3803,22 +3747,22 @@
         <v>9</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>372</v>
+        <v>367</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>373</v>
+        <v>368</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6">
@@ -3829,22 +3773,22 @@
         <v>12</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>374</v>
+        <v>369</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>375</v>
+        <v>370</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>372</v>
+        <v>367</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>376</v>
+        <v>371</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7">
@@ -3852,25 +3796,25 @@
         <v>14</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>377</v>
+        <v>372</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>378</v>
+        <v>373</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>375</v>
+        <v>370</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>372</v>
+        <v>367</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>369</v>
+        <v>364</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>379</v>
+        <v>374</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8">
@@ -3880,23 +3824,23 @@
       <c r="B8" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="3" t="s">
-        <v>192</v>
+      <c r="C8" s="2" t="s">
+        <v>375</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>375</v>
+        <v>156</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>372</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>380</v>
+        <v>367</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>185</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>381</v>
+        <v>376</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9">
@@ -3907,22 +3851,22 @@
         <v>21</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>375</v>
+        <v>156</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>372</v>
+        <v>156</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>382</v>
+        <v>377</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>383</v>
+        <v>378</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10">
@@ -3930,51 +3874,51 @@
         <v>23</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>24</v>
+        <v>379</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>384</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>162</v>
+        <v>380</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>185</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>372</v>
+        <v>381</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>35</v>
+        <v>383</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>26</v>
+        <v>384</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>27</v>
+        <v>385</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>162</v>
+        <v>386</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>162</v>
+        <v>387</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12">
@@ -3982,753 +3926,701 @@
         <v>29</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>388</v>
+        <v>29</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>389</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>192</v>
+        <v>29</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>29</v>
       </c>
       <c r="E12" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="s">
         <v>390</v>
       </c>
-      <c r="F12" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>391</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>392</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="s">
-        <v>393</v>
-      </c>
       <c r="B13" s="2" t="s">
-        <v>394</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>192</v>
+        <v>29</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>29</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>395</v>
+        <v>29</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>396</v>
+        <v>29</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>397</v>
+        <v>29</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>398</v>
+        <v>29</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="s">
-        <v>399</v>
+      <c r="A15" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>35</v>
+        <v>370</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>185</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>35</v>
+        <v>367</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>185</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>35</v>
+        <v>391</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>35</v>
+        <v>392</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>35</v>
+        <v>393</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>35</v>
+        <v>394</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>185</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>35</v>
+        <v>364</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>185</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>35</v>
+        <v>395</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>35</v>
+        <v>396</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="s">
-        <v>37</v>
+        <v>397</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>375</v>
+        <v>41</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>185</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>372</v>
+        <v>185</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>185</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>400</v>
+        <v>185</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>185</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>401</v>
+        <v>29</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="s">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>402</v>
+        <v>29</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>403</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>192</v>
+        <v>29</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>29</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>369</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>192</v>
+        <v>29</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>29</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>404</v>
+        <v>29</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>405</v>
+        <v>29</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="s">
-        <v>406</v>
+        <v>398</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>192</v>
+        <v>44</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>399</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>192</v>
+        <v>185</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>364</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="G19" s="3" t="s">
-        <v>192</v>
+        <v>185</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>400</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>35</v>
+        <v>401</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="s">
-        <v>35</v>
+        <v>402</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>35</v>
+        <v>403</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>185</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>35</v>
+        <v>404</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>35</v>
+        <v>405</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>35</v>
+        <v>406</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>35</v>
+        <v>407</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="s">
-        <v>407</v>
+        <v>29</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>408</v>
-      </c>
-      <c r="D21" s="3" t="s">
-        <v>192</v>
+        <v>29</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>29</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>369</v>
-      </c>
-      <c r="F21" s="3" t="s">
-        <v>192</v>
+        <v>29</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>29</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>409</v>
+        <v>29</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>410</v>
+        <v>29</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>412</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>192</v>
+        <v>29</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>29</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>413</v>
+        <v>29</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>414</v>
+        <v>29</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>415</v>
+        <v>29</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>416</v>
+        <v>29</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="s">
-        <v>35</v>
+        <v>409</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>35</v>
+        <v>410</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>35</v>
+        <v>104</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>35</v>
+        <v>411</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>35</v>
+        <v>412</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>185</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>35</v>
+        <v>413</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>35</v>
+        <v>401</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="D24" s="2" t="s">
         <v>417</v>
       </c>
-      <c r="B24" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>35</v>
-      </c>
       <c r="E24" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>35</v>
+        <v>417</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>185</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>35</v>
+        <v>416</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>35</v>
+        <v>418</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>420</v>
+        <v>411</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>421</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>422</v>
+        <v>104</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>410</v>
+        <v>401</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="s">
-        <v>423</v>
+        <v>29</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>424</v>
+        <v>29</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>425</v>
+        <v>29</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>426</v>
+        <v>29</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>426</v>
-      </c>
-      <c r="F26" s="3" t="s">
-        <v>192</v>
+        <v>29</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>29</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>425</v>
+        <v>29</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>427</v>
+        <v>29</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="s">
-        <v>428</v>
+        <v>422</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>429</v>
+        <v>29</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>110</v>
+        <v>29</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>420</v>
+        <v>29</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>430</v>
-      </c>
-      <c r="F27" s="3" t="s">
-        <v>192</v>
+        <v>29</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>29</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>110</v>
+        <v>423</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>410</v>
+        <v>424</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="s">
-        <v>431</v>
+      <c r="A29" s="3" t="s">
+        <v>425</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>432</v>
+        <v>29</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>433</v>
+        <v>29</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="s">
-        <v>434</v>
+      <c r="A31" s="2" t="s">
+        <v>426</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>35</v>
+        <v>427</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>185</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>35</v>
+        <v>386</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>35</v>
+        <v>428</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>35</v>
+        <v>429</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>35</v>
+        <v>430</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="s">
-        <v>35</v>
+        <v>398</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>35</v>
+        <v>431</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>35</v>
+        <v>432</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>185</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F32" s="2" t="s">
-        <v>35</v>
+        <v>364</v>
+      </c>
+      <c r="F32" s="3" t="s">
+        <v>185</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>35</v>
+        <v>433</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>35</v>
+        <v>434</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="s">
-        <v>435</v>
+        <v>402</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>436</v>
+        <v>403</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>395</v>
+        <v>404</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>437</v>
+        <v>405</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>438</v>
+        <v>406</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>439</v>
+        <v>407</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="s">
-        <v>407</v>
+        <v>29</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>440</v>
+        <v>29</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>441</v>
-      </c>
-      <c r="D34" s="3" t="s">
-        <v>192</v>
+        <v>29</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>29</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>369</v>
-      </c>
-      <c r="F34" s="3" t="s">
-        <v>192</v>
+        <v>29</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>29</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>442</v>
+        <v>29</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>443</v>
+        <v>29</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="s">
-        <v>411</v>
+        <v>435</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>412</v>
-      </c>
-      <c r="C35" s="3" t="s">
-        <v>192</v>
+        <v>29</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>29</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>413</v>
+        <v>29</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>414</v>
+        <v>29</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>415</v>
+        <v>29</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>416</v>
+        <v>29</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="s">
-        <v>35</v>
+        <v>436</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="s">
-        <v>444</v>
+        <v>29</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="s">
-        <v>445</v>
+        <v>437</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>35</v>
+        <v>438</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D39" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="E39" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F39" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="G39" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="H39" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="s">
-        <v>446</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="E40" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F40" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="G40" s="2" t="s">
-        <v>447</v>
-      </c>
-      <c r="H40" s="2" t="s">
-        <v>433</v>
+        <v>424</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix days of week in itinerary (was off by 2)
</commit_message>
<xml_diff>
--- a/europe_nyc_trip_plan.xlsx
+++ b/europe_nyc_trip_plan.xlsx
@@ -3,21 +3,21 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr date1904="false"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Itinerary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Flights" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Ferries" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Accommodation" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Budget" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Daily Costs (2 ppl)" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Itinerary" sheetId="7" state="visible" r:id="rId6"/>
+    <sheet name="Flights" sheetId="2" state="visible" r:id="rId1"/>
+    <sheet name="Ferries" sheetId="3" state="visible" r:id="rId2"/>
+    <sheet name="Accommodation" sheetId="4" state="visible" r:id="rId3"/>
+    <sheet name="Budget" sheetId="5" state="visible" r:id="rId4"/>
+    <sheet name="Daily Costs (2 ppl)" sheetId="6" state="visible" r:id="rId5"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="227">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -689,6 +689,15 @@
   </si>
   <si>
     <t xml:space="preserve">$210-380</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sun-Mon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mon-Fri</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sat-Thu</t>
   </si>
 </sst>
 </file>
@@ -1017,420 +1026,6 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="9.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="7.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="40.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="66.71" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="14.71" hidden="0" customWidth="1"/>
-    <col min="6" max="6" width="9.15" hidden="0" customWidth="1"/>
-    <col min="7" max="7" width="9.15" hidden="0" customWidth="1"/>
-    <col min="8" max="8" width="9.15" hidden="0" customWidth="1"/>
-    <col min="9" max="9" width="9.15" hidden="0" customWidth="1"/>
-    <col min="10" max="10" width="9.15" hidden="0" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B5" t="s">
-        <v>19</v>
-      </c>
-      <c r="C5" t="s">
-        <v>20</v>
-      </c>
-      <c r="D5" t="s">
-        <v>21</v>
-      </c>
-      <c r="E5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C6" t="s">
-        <v>23</v>
-      </c>
-      <c r="D6" t="s">
-        <v>24</v>
-      </c>
-      <c r="E6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s">
-        <v>25</v>
-      </c>
-      <c r="B7" t="s">
-        <v>26</v>
-      </c>
-      <c r="C7" t="s">
-        <v>27</v>
-      </c>
-      <c r="D7" t="s">
-        <v>28</v>
-      </c>
-      <c r="E7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s">
-        <v>29</v>
-      </c>
-      <c r="B8" t="s">
-        <v>30</v>
-      </c>
-      <c r="C8" t="s">
-        <v>27</v>
-      </c>
-      <c r="D8" t="s">
-        <v>31</v>
-      </c>
-      <c r="E8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s">
-        <v>32</v>
-      </c>
-      <c r="B9" t="s">
-        <v>33</v>
-      </c>
-      <c r="C9" t="s">
-        <v>27</v>
-      </c>
-      <c r="D9" t="s">
-        <v>34</v>
-      </c>
-      <c r="E9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="s">
-        <v>35</v>
-      </c>
-      <c r="B10" t="s">
-        <v>36</v>
-      </c>
-      <c r="C10" t="s">
-        <v>27</v>
-      </c>
-      <c r="D10" t="s">
-        <v>37</v>
-      </c>
-      <c r="E10" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="s">
-        <v>38</v>
-      </c>
-      <c r="B11" t="s">
-        <v>11</v>
-      </c>
-      <c r="C11" t="s">
-        <v>39</v>
-      </c>
-      <c r="D11" t="s">
-        <v>40</v>
-      </c>
-      <c r="E11" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="s">
-        <v>41</v>
-      </c>
-      <c r="B12" t="s">
-        <v>16</v>
-      </c>
-      <c r="C12" t="s">
-        <v>42</v>
-      </c>
-      <c r="D12" t="s">
-        <v>43</v>
-      </c>
-      <c r="E12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="s">
-        <v>44</v>
-      </c>
-      <c r="B13" t="s">
-        <v>19</v>
-      </c>
-      <c r="C13" t="s">
-        <v>45</v>
-      </c>
-      <c r="D13" t="s">
-        <v>46</v>
-      </c>
-      <c r="E13" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="s">
-        <v>48</v>
-      </c>
-      <c r="B14" t="s">
-        <v>26</v>
-      </c>
-      <c r="C14" t="s">
-        <v>49</v>
-      </c>
-      <c r="D14" t="s">
-        <v>50</v>
-      </c>
-      <c r="E14" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="s">
-        <v>51</v>
-      </c>
-      <c r="B15" t="s">
-        <v>30</v>
-      </c>
-      <c r="C15" t="s">
-        <v>49</v>
-      </c>
-      <c r="D15" t="s">
-        <v>52</v>
-      </c>
-      <c r="E15" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="s">
-        <v>53</v>
-      </c>
-      <c r="B16" t="s">
-        <v>33</v>
-      </c>
-      <c r="C16" t="s">
-        <v>54</v>
-      </c>
-      <c r="D16" t="s">
-        <v>55</v>
-      </c>
-      <c r="E16" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="s">
-        <v>57</v>
-      </c>
-      <c r="B17" t="s">
-        <v>58</v>
-      </c>
-      <c r="C17" t="s">
-        <v>59</v>
-      </c>
-      <c r="D17" t="s">
-        <v>60</v>
-      </c>
-      <c r="E17" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="s">
-        <v>62</v>
-      </c>
-      <c r="B18" t="s">
-        <v>30</v>
-      </c>
-      <c r="C18" t="s">
-        <v>63</v>
-      </c>
-      <c r="D18" t="s">
-        <v>64</v>
-      </c>
-      <c r="E18" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="s">
-        <v>65</v>
-      </c>
-      <c r="B19" t="s">
-        <v>66</v>
-      </c>
-      <c r="C19" t="s">
-        <v>67</v>
-      </c>
-      <c r="D19" t="s">
-        <v>68</v>
-      </c>
-      <c r="E19" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="s">
-        <v>70</v>
-      </c>
-      <c r="B20" t="s">
-        <v>26</v>
-      </c>
-      <c r="C20" t="s">
-        <v>71</v>
-      </c>
-      <c r="D20" t="s">
-        <v>72</v>
-      </c>
-      <c r="E20" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="s">
-        <v>73</v>
-      </c>
-      <c r="B21" t="s">
-        <v>66</v>
-      </c>
-      <c r="C21" t="s">
-        <v>74</v>
-      </c>
-      <c r="D21" t="s">
-        <v>75</v>
-      </c>
-      <c r="E21" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="s">
-        <v>76</v>
-      </c>
-      <c r="B22" t="s">
-        <v>26</v>
-      </c>
-      <c r="C22" t="s">
-        <v>77</v>
-      </c>
-      <c r="D22" t="s">
-        <v>78</v>
-      </c>
-      <c r="E22" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="s">
-        <v>80</v>
-      </c>
-      <c r="B23" t="s">
-        <v>30</v>
-      </c>
-      <c r="C23" t="s">
-        <v>81</v>
-      </c>
-      <c r="D23" t="s">
-        <v>82</v>
-      </c>
-      <c r="E23" t="s">
-        <v>9</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
-  <cols>
     <col min="1" max="1" width="29.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="9.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="38.71" hidden="0" customWidth="1"/>
@@ -1649,7 +1244,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
@@ -1732,7 +1327,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
@@ -1915,7 +1510,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
@@ -2078,7 +1673,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
@@ -2283,4 +1878,413 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
+    <col min="1" max="1" width="9.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="7.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="40.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="66.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="14.71" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>224</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" t="s">
+        <v>28</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" t="s">
+        <v>31</v>
+      </c>
+      <c r="E8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" t="s">
+        <v>37</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>38</v>
+      </c>
+      <c r="B11" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" t="s">
+        <v>39</v>
+      </c>
+      <c r="D11" t="s">
+        <v>40</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>41</v>
+      </c>
+      <c r="B12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" t="s">
+        <v>42</v>
+      </c>
+      <c r="D12" t="s">
+        <v>43</v>
+      </c>
+      <c r="E12" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>44</v>
+      </c>
+      <c r="B13" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13" t="s">
+        <v>45</v>
+      </c>
+      <c r="D13" t="s">
+        <v>46</v>
+      </c>
+      <c r="E13" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>48</v>
+      </c>
+      <c r="B14" t="s">
+        <v>30</v>
+      </c>
+      <c r="C14" t="s">
+        <v>49</v>
+      </c>
+      <c r="D14" t="s">
+        <v>50</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>51</v>
+      </c>
+      <c r="B15" t="s">
+        <v>33</v>
+      </c>
+      <c r="C15" t="s">
+        <v>49</v>
+      </c>
+      <c r="D15" t="s">
+        <v>52</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>53</v>
+      </c>
+      <c r="B16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C16" t="s">
+        <v>54</v>
+      </c>
+      <c r="D16" t="s">
+        <v>55</v>
+      </c>
+      <c r="E16" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>57</v>
+      </c>
+      <c r="B17" t="s">
+        <v>225</v>
+      </c>
+      <c r="C17" t="s">
+        <v>59</v>
+      </c>
+      <c r="D17" t="s">
+        <v>60</v>
+      </c>
+      <c r="E17" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>62</v>
+      </c>
+      <c r="B18" t="s">
+        <v>33</v>
+      </c>
+      <c r="C18" t="s">
+        <v>63</v>
+      </c>
+      <c r="D18" t="s">
+        <v>64</v>
+      </c>
+      <c r="E18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>65</v>
+      </c>
+      <c r="B19" t="s">
+        <v>226</v>
+      </c>
+      <c r="C19" t="s">
+        <v>67</v>
+      </c>
+      <c r="D19" t="s">
+        <v>68</v>
+      </c>
+      <c r="E19" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>70</v>
+      </c>
+      <c r="B20" t="s">
+        <v>30</v>
+      </c>
+      <c r="C20" t="s">
+        <v>71</v>
+      </c>
+      <c r="D20" t="s">
+        <v>72</v>
+      </c>
+      <c r="E20" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>73</v>
+      </c>
+      <c r="B21" t="s">
+        <v>226</v>
+      </c>
+      <c r="C21" t="s">
+        <v>74</v>
+      </c>
+      <c r="D21" t="s">
+        <v>75</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>76</v>
+      </c>
+      <c r="B22" t="s">
+        <v>30</v>
+      </c>
+      <c r="C22" t="s">
+        <v>77</v>
+      </c>
+      <c r="D22" t="s">
+        <v>78</v>
+      </c>
+      <c r="E22" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>80</v>
+      </c>
+      <c r="B23" t="s">
+        <v>33</v>
+      </c>
+      <c r="C23" t="s">
+        <v>81</v>
+      </c>
+      <c r="D23" t="s">
+        <v>82</v>
+      </c>
+      <c r="E23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Change outbound flight to May 25 evening departure
</commit_message>
<xml_diff>
--- a/europe_nyc_trip_plan.xlsx
+++ b/europe_nyc_trip_plan.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr date1904="false"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Itinerary" sheetId="7" state="visible" r:id="rId6"/>
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="230">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -698,6 +698,15 @@
   </si>
   <si>
     <t xml:space="preserve">Sat-Thu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">May 25-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mon-Tue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fly LAX &gt; Florence (evening departure, arrive next day)</t>
   </si>
 </sst>
 </file>
@@ -1911,16 +1920,16 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>227</v>
       </c>
       <c r="B2" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="C2" t="s">
         <v>7</v>
       </c>
       <c r="D2" t="s">
-        <v>8</v>
+        <v>229</v>
       </c>
       <c r="E2" t="s">
         <v>9</v>

</xml_diff>

<commit_message>
Switch Naxos to Paros
</commit_message>
<xml_diff>
--- a/europe_nyc_trip_plan.xlsx
+++ b/europe_nyc_trip_plan.xlsx
@@ -6,18 +6,18 @@
     <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
-    <sheet name="Itinerary" sheetId="7" state="visible" r:id="rId6"/>
-    <sheet name="Flights" sheetId="2" state="visible" r:id="rId1"/>
-    <sheet name="Ferries" sheetId="3" state="visible" r:id="rId2"/>
-    <sheet name="Accommodation" sheetId="4" state="visible" r:id="rId3"/>
-    <sheet name="Budget" sheetId="5" state="visible" r:id="rId4"/>
-    <sheet name="Daily Costs (2 ppl)" sheetId="6" state="visible" r:id="rId5"/>
+    <sheet name="Itinerary" sheetId="7" state="visible" r:id="rId1"/>
+    <sheet name="Flights" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Ferries" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Accommodation" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Budget" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Daily Costs (2 ppl)" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="240">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -707,6 +707,36 @@
   </si>
   <si>
     <t xml:space="preserve">Fly LAX &gt; Florence (evening departure, arrive next day)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paros</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ferry from Piraeus (~5h), arrive Paros afternoon, explore Chora</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Naoussa &amp; coastal paths: Halki, Filoti, Apiranthos. Kitron tasting</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paros &gt; Athens &gt; Zagreb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Athens (Piraeus) &gt; Paros</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Depart Piraeus morning, arrive Paros early afternoon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paros &gt; Athens (Piraeus)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Depart Paros early morning (~7am), arrive Piraeus ~10:30-12:30pm. Catch afternoon flight to Zagreb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paros Town (Chora) or inland near Halki, 1 room 1 bed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 ferry rides Athens-Paros round trip</t>
   </si>
 </sst>
 </file>
@@ -1035,6 +1065,415 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
+    <col min="1" max="1" width="9.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="7.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="40.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="66.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="14.71" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>227</v>
+      </c>
+      <c r="B2" t="s">
+        <v>228</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" t="s">
+        <v>229</v>
+      </c>
+      <c r="E2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" t="s">
+        <v>230</v>
+      </c>
+      <c r="D7" t="s">
+        <v>231</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" t="s">
+        <v>230</v>
+      </c>
+      <c r="D8" t="s">
+        <v>31</v>
+      </c>
+      <c r="E8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" t="s">
+        <v>230</v>
+      </c>
+      <c r="D9" t="s">
+        <v>232</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" t="s">
+        <v>230</v>
+      </c>
+      <c r="D10" t="s">
+        <v>37</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>38</v>
+      </c>
+      <c r="B11" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" t="s">
+        <v>233</v>
+      </c>
+      <c r="D11" t="s">
+        <v>40</v>
+      </c>
+      <c r="E11" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>41</v>
+      </c>
+      <c r="B12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" t="s">
+        <v>42</v>
+      </c>
+      <c r="D12" t="s">
+        <v>43</v>
+      </c>
+      <c r="E12" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>44</v>
+      </c>
+      <c r="B13" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13" t="s">
+        <v>45</v>
+      </c>
+      <c r="D13" t="s">
+        <v>46</v>
+      </c>
+      <c r="E13" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>48</v>
+      </c>
+      <c r="B14" t="s">
+        <v>30</v>
+      </c>
+      <c r="C14" t="s">
+        <v>49</v>
+      </c>
+      <c r="D14" t="s">
+        <v>50</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>51</v>
+      </c>
+      <c r="B15" t="s">
+        <v>33</v>
+      </c>
+      <c r="C15" t="s">
+        <v>49</v>
+      </c>
+      <c r="D15" t="s">
+        <v>52</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>53</v>
+      </c>
+      <c r="B16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C16" t="s">
+        <v>54</v>
+      </c>
+      <c r="D16" t="s">
+        <v>55</v>
+      </c>
+      <c r="E16" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>57</v>
+      </c>
+      <c r="B17" t="s">
+        <v>225</v>
+      </c>
+      <c r="C17" t="s">
+        <v>59</v>
+      </c>
+      <c r="D17" t="s">
+        <v>60</v>
+      </c>
+      <c r="E17" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>62</v>
+      </c>
+      <c r="B18" t="s">
+        <v>33</v>
+      </c>
+      <c r="C18" t="s">
+        <v>63</v>
+      </c>
+      <c r="D18" t="s">
+        <v>64</v>
+      </c>
+      <c r="E18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>65</v>
+      </c>
+      <c r="B19" t="s">
+        <v>226</v>
+      </c>
+      <c r="C19" t="s">
+        <v>67</v>
+      </c>
+      <c r="D19" t="s">
+        <v>68</v>
+      </c>
+      <c r="E19" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>70</v>
+      </c>
+      <c r="B20" t="s">
+        <v>30</v>
+      </c>
+      <c r="C20" t="s">
+        <v>71</v>
+      </c>
+      <c r="D20" t="s">
+        <v>72</v>
+      </c>
+      <c r="E20" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>73</v>
+      </c>
+      <c r="B21" t="s">
+        <v>226</v>
+      </c>
+      <c r="C21" t="s">
+        <v>74</v>
+      </c>
+      <c r="D21" t="s">
+        <v>75</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>76</v>
+      </c>
+      <c r="B22" t="s">
+        <v>30</v>
+      </c>
+      <c r="C22" t="s">
+        <v>77</v>
+      </c>
+      <c r="D22" t="s">
+        <v>78</v>
+      </c>
+      <c r="E22" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>80</v>
+      </c>
+      <c r="B23" t="s">
+        <v>33</v>
+      </c>
+      <c r="C23" t="s">
+        <v>81</v>
+      </c>
+      <c r="D23" t="s">
+        <v>82</v>
+      </c>
+      <c r="E23" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
     <col min="1" max="1" width="29.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="9.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="38.71" hidden="0" customWidth="1"/>
@@ -1253,7 +1692,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
@@ -1292,7 +1731,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>128</v>
+        <v>234</v>
       </c>
       <c r="B2" t="s">
         <v>25</v>
@@ -1307,12 +1746,12 @@
         <v>131</v>
       </c>
       <c r="F2" t="s">
-        <v>132</v>
+        <v>235</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>133</v>
+        <v>236</v>
       </c>
       <c r="B3" t="s">
         <v>38</v>
@@ -1327,7 +1766,7 @@
         <v>131</v>
       </c>
       <c r="F3" t="s">
-        <v>134</v>
+        <v>237</v>
       </c>
     </row>
   </sheetData>
@@ -1336,7 +1775,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
@@ -1415,7 +1854,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>27</v>
+        <v>230</v>
       </c>
       <c r="B4" t="n">
         <v>3</v>
@@ -1430,7 +1869,7 @@
         <v>147</v>
       </c>
       <c r="F4" t="s">
-        <v>148</v>
+        <v>238</v>
       </c>
     </row>
     <row r="5">
@@ -1519,7 +1958,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
@@ -1575,7 +2014,7 @@
         <v>174</v>
       </c>
       <c r="D3" t="s">
-        <v>175</v>
+        <v>239</v>
       </c>
     </row>
     <row r="4">
@@ -1682,7 +2121,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
@@ -1770,7 +2209,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>27</v>
+        <v>230</v>
       </c>
       <c r="B4" t="n">
         <v>4</v>
@@ -1881,415 +2320,6 @@
       </c>
       <c r="G8" t="s">
         <v>223</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
-  <cols>
-    <col min="1" max="1" width="9.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="7.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="40.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="66.71" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="14.71" hidden="0" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s">
-        <v>227</v>
-      </c>
-      <c r="B2" t="s">
-        <v>228</v>
-      </c>
-      <c r="C2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" t="s">
-        <v>229</v>
-      </c>
-      <c r="E2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B5" t="s">
-        <v>26</v>
-      </c>
-      <c r="C5" t="s">
-        <v>20</v>
-      </c>
-      <c r="D5" t="s">
-        <v>21</v>
-      </c>
-      <c r="E5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B6" t="s">
-        <v>26</v>
-      </c>
-      <c r="C6" t="s">
-        <v>23</v>
-      </c>
-      <c r="D6" t="s">
-        <v>24</v>
-      </c>
-      <c r="E6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s">
-        <v>25</v>
-      </c>
-      <c r="B7" t="s">
-        <v>30</v>
-      </c>
-      <c r="C7" t="s">
-        <v>27</v>
-      </c>
-      <c r="D7" t="s">
-        <v>28</v>
-      </c>
-      <c r="E7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s">
-        <v>29</v>
-      </c>
-      <c r="B8" t="s">
-        <v>33</v>
-      </c>
-      <c r="C8" t="s">
-        <v>27</v>
-      </c>
-      <c r="D8" t="s">
-        <v>31</v>
-      </c>
-      <c r="E8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s">
-        <v>32</v>
-      </c>
-      <c r="B9" t="s">
-        <v>36</v>
-      </c>
-      <c r="C9" t="s">
-        <v>27</v>
-      </c>
-      <c r="D9" t="s">
-        <v>34</v>
-      </c>
-      <c r="E9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="s">
-        <v>35</v>
-      </c>
-      <c r="B10" t="s">
-        <v>11</v>
-      </c>
-      <c r="C10" t="s">
-        <v>27</v>
-      </c>
-      <c r="D10" t="s">
-        <v>37</v>
-      </c>
-      <c r="E10" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="s">
-        <v>38</v>
-      </c>
-      <c r="B11" t="s">
-        <v>16</v>
-      </c>
-      <c r="C11" t="s">
-        <v>39</v>
-      </c>
-      <c r="D11" t="s">
-        <v>40</v>
-      </c>
-      <c r="E11" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="s">
-        <v>41</v>
-      </c>
-      <c r="B12" t="s">
-        <v>19</v>
-      </c>
-      <c r="C12" t="s">
-        <v>42</v>
-      </c>
-      <c r="D12" t="s">
-        <v>43</v>
-      </c>
-      <c r="E12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="s">
-        <v>44</v>
-      </c>
-      <c r="B13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C13" t="s">
-        <v>45</v>
-      </c>
-      <c r="D13" t="s">
-        <v>46</v>
-      </c>
-      <c r="E13" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="s">
-        <v>48</v>
-      </c>
-      <c r="B14" t="s">
-        <v>30</v>
-      </c>
-      <c r="C14" t="s">
-        <v>49</v>
-      </c>
-      <c r="D14" t="s">
-        <v>50</v>
-      </c>
-      <c r="E14" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="s">
-        <v>51</v>
-      </c>
-      <c r="B15" t="s">
-        <v>33</v>
-      </c>
-      <c r="C15" t="s">
-        <v>49</v>
-      </c>
-      <c r="D15" t="s">
-        <v>52</v>
-      </c>
-      <c r="E15" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="s">
-        <v>53</v>
-      </c>
-      <c r="B16" t="s">
-        <v>36</v>
-      </c>
-      <c r="C16" t="s">
-        <v>54</v>
-      </c>
-      <c r="D16" t="s">
-        <v>55</v>
-      </c>
-      <c r="E16" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="s">
-        <v>57</v>
-      </c>
-      <c r="B17" t="s">
-        <v>225</v>
-      </c>
-      <c r="C17" t="s">
-        <v>59</v>
-      </c>
-      <c r="D17" t="s">
-        <v>60</v>
-      </c>
-      <c r="E17" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="s">
-        <v>62</v>
-      </c>
-      <c r="B18" t="s">
-        <v>33</v>
-      </c>
-      <c r="C18" t="s">
-        <v>63</v>
-      </c>
-      <c r="D18" t="s">
-        <v>64</v>
-      </c>
-      <c r="E18" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="s">
-        <v>65</v>
-      </c>
-      <c r="B19" t="s">
-        <v>226</v>
-      </c>
-      <c r="C19" t="s">
-        <v>67</v>
-      </c>
-      <c r="D19" t="s">
-        <v>68</v>
-      </c>
-      <c r="E19" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="s">
-        <v>70</v>
-      </c>
-      <c r="B20" t="s">
-        <v>30</v>
-      </c>
-      <c r="C20" t="s">
-        <v>71</v>
-      </c>
-      <c r="D20" t="s">
-        <v>72</v>
-      </c>
-      <c r="E20" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="s">
-        <v>73</v>
-      </c>
-      <c r="B21" t="s">
-        <v>226</v>
-      </c>
-      <c r="C21" t="s">
-        <v>74</v>
-      </c>
-      <c r="D21" t="s">
-        <v>75</v>
-      </c>
-      <c r="E21" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="s">
-        <v>76</v>
-      </c>
-      <c r="B22" t="s">
-        <v>30</v>
-      </c>
-      <c r="C22" t="s">
-        <v>77</v>
-      </c>
-      <c r="D22" t="s">
-        <v>78</v>
-      </c>
-      <c r="E22" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="s">
-        <v>80</v>
-      </c>
-      <c r="B23" t="s">
-        <v>33</v>
-      </c>
-      <c r="C23" t="s">
-        <v>81</v>
-      </c>
-      <c r="D23" t="s">
-        <v>82</v>
-      </c>
-      <c r="E23" t="s">
-        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Keep London arrival Jun 7, extra day goes to Zagreb
</commit_message>
<xml_diff>
--- a/europe_nyc_trip_plan.xlsx
+++ b/europe_nyc_trip_plan.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="217">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -148,7 +148,7 @@
     <t xml:space="preserve">Zagreb</t>
   </si>
   <si>
-    <t xml:space="preserve">Explore Zagreb Upper Town, food scene</t>
+    <t xml:space="preserve">Explore Zagreb Upper Town, Dolac Market, food scene</t>
   </si>
   <si>
     <t xml:space="preserve">Jun 3</t>
@@ -187,22 +187,16 @@
     <t xml:space="preserve">Jun 7</t>
   </si>
   <si>
-    <t xml:space="preserve">Elafiti islands day trip or Cavtat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jun 8</t>
-  </si>
-  <si>
     <t xml:space="preserve">Dubrovnik &gt; London</t>
   </si>
   <si>
     <t xml:space="preserve">Fly Dubrovnik &gt; London Gatwick (easyJet)</t>
   </si>
   <si>
-    <t xml:space="preserve">Jun 8-12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mon-Fri</t>
+    <t xml:space="preserve">Jun 7-12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sun-Fri</t>
   </si>
   <si>
     <t xml:space="preserve">London</t>
@@ -211,7 +205,7 @@
     <t xml:space="preserve">Free accommodation, explore London</t>
   </si>
   <si>
-    <t xml:space="preserve">Yes (x5)</t>
+    <t xml:space="preserve">Yes (x6)</t>
   </si>
   <si>
     <t xml:space="preserve">Jun 13</t>
@@ -253,9 +247,6 @@
     <t xml:space="preserve">NYC exploring, 1 room 1 bed</t>
   </si>
   <si>
-    <t xml:space="preserve">Yes (x6)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Jun 26</t>
   </si>
   <si>
@@ -463,13 +454,13 @@
     <t xml:space="preserve">Athens (return)</t>
   </si>
   <si>
-    <t xml:space="preserve">May 31 (after ferry back)</t>
+    <t xml:space="preserve">May 31 (after ferry)</t>
   </si>
   <si>
     <t xml:space="preserve">$60-100</t>
   </si>
   <si>
-    <t xml:space="preserve">Jun 1-2 (arrive Mon evening)</t>
+    <t xml:space="preserve">Jun 1-3 (arrive Mon evening)</t>
   </si>
   <si>
     <t xml:space="preserve">$80-140</t>
@@ -481,7 +472,7 @@
     <t xml:space="preserve">Free</t>
   </si>
   <si>
-    <t xml:space="preserve">Jun 8-12 (free accommodation)</t>
+    <t xml:space="preserve">Jun 7-12 (free)</t>
   </si>
   <si>
     <t xml:space="preserve">$150-250</t>
@@ -523,16 +514,16 @@
     <t xml:space="preserve">2 ferries x 2 people</t>
   </si>
   <si>
-    <t xml:space="preserve">Accommodation (17 paid nights)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$1,800</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$3,200</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2 Florence + 1 Athens + 2 Paros + 1 Athens return + 2 Zagreb + 3 Dubrovnik + 6 NYC</t>
+    <t xml:space="preserve">Accommodation (18 paid nights)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$1,860</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$3,300</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 Florence + 1 Athens + 2 Paros + 1 Athens return + 3 Zagreb + 3 Dubrovnik + 6 NYC</t>
   </si>
   <si>
     <t xml:space="preserve">Food &amp; Drink</t>
@@ -577,10 +568,10 @@
     <t xml:space="preserve">TOTAL (2 people)</t>
   </si>
   <si>
-    <t xml:space="preserve">$6,680</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$11,800</t>
+    <t xml:space="preserve">$6,740</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$11,900</t>
   </si>
   <si>
     <t xml:space="preserve">For 2 people total</t>
@@ -643,7 +634,10 @@
     <t xml:space="preserve">Overnight before Zagreb flight</t>
   </si>
   <si>
-    <t xml:space="preserve">Upper Town, food markets</t>
+    <t xml:space="preserve">3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Upper Town, Dolac Market, food scene</t>
   </si>
   <si>
     <t xml:space="preserve">Plitvice entrance</t>
@@ -661,22 +655,16 @@
     <t xml:space="preserve">Park entrance ~$25/pp, bus ~$15-18/pp each way</t>
   </si>
   <si>
-    <t xml:space="preserve">3</t>
-  </si>
-  <si>
     <t xml:space="preserve">$15-30</t>
   </si>
   <si>
     <t xml:space="preserve">Walls ticket ~$35, Lokrum ferry ~$15</t>
   </si>
   <si>
-    <t xml:space="preserve">5</t>
+    <t xml:space="preserve">6</t>
   </si>
   <si>
     <t xml:space="preserve">Free accommodation helps a lot</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6</t>
   </si>
   <si>
     <t xml:space="preserve">1 room 1 bed for 2 ppl</t>
@@ -1278,61 +1266,61 @@
         <v>33</v>
       </c>
       <c r="C16" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="D16" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E16" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B17" t="s">
-        <v>38</v>
+        <v>59</v>
       </c>
       <c r="C17" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D17" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="E17" t="s">
-        <v>9</v>
+        <v>62</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B18" t="s">
-        <v>61</v>
+        <v>30</v>
       </c>
       <c r="C18" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D18" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E18" t="s">
-        <v>64</v>
+        <v>9</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B19" t="s">
-        <v>30</v>
+        <v>67</v>
       </c>
       <c r="C19" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D19" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E19" t="s">
         <v>9</v>
@@ -1340,16 +1328,16 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B20" t="s">
-        <v>69</v>
+        <v>26</v>
       </c>
       <c r="C20" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D20" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E20" t="s">
         <v>9</v>
@@ -1357,36 +1345,36 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B21" t="s">
-        <v>26</v>
+        <v>67</v>
       </c>
       <c r="C21" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D21" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E21" t="s">
-        <v>9</v>
+        <v>62</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B22" t="s">
-        <v>69</v>
+        <v>26</v>
       </c>
       <c r="C22" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D22" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E22" t="s">
-        <v>78</v>
+        <v>9</v>
       </c>
     </row>
     <row r="23">
@@ -1394,7 +1382,7 @@
         <v>79</v>
       </c>
       <c r="B23" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="C23" t="s">
         <v>80</v>
@@ -1403,23 +1391,6 @@
         <v>81</v>
       </c>
       <c r="E23" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="s">
-        <v>82</v>
-      </c>
-      <c r="B24" t="s">
-        <v>30</v>
-      </c>
-      <c r="C24" t="s">
-        <v>83</v>
-      </c>
-      <c r="D24" t="s">
-        <v>84</v>
-      </c>
-      <c r="E24" t="s">
         <v>9</v>
       </c>
     </row>
@@ -1444,42 +1415,42 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
       </c>
       <c r="C1" t="s">
+        <v>83</v>
+      </c>
+      <c r="D1" t="s">
+        <v>84</v>
+      </c>
+      <c r="E1" t="s">
+        <v>85</v>
+      </c>
+      <c r="F1" t="s">
         <v>86</v>
-      </c>
-      <c r="D1" t="s">
-        <v>87</v>
-      </c>
-      <c r="E1" t="s">
-        <v>88</v>
-      </c>
-      <c r="F1" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D2" t="s">
         <v>90</v>
       </c>
-      <c r="B2" t="s">
+      <c r="E2" t="s">
         <v>91</v>
       </c>
-      <c r="C2" t="s">
+      <c r="F2" t="s">
         <v>92</v>
-      </c>
-      <c r="D2" t="s">
-        <v>93</v>
-      </c>
-      <c r="E2" t="s">
-        <v>94</v>
-      </c>
-      <c r="F2" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="3">
@@ -1490,16 +1461,16 @@
         <v>18</v>
       </c>
       <c r="C3" t="s">
+        <v>93</v>
+      </c>
+      <c r="D3" t="s">
+        <v>94</v>
+      </c>
+      <c r="E3" t="s">
+        <v>95</v>
+      </c>
+      <c r="F3" t="s">
         <v>96</v>
-      </c>
-      <c r="D3" t="s">
-        <v>97</v>
-      </c>
-      <c r="E3" t="s">
-        <v>98</v>
-      </c>
-      <c r="F3" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="4">
@@ -1510,16 +1481,16 @@
         <v>41</v>
       </c>
       <c r="C4" t="s">
+        <v>97</v>
+      </c>
+      <c r="D4" t="s">
+        <v>98</v>
+      </c>
+      <c r="E4" t="s">
+        <v>99</v>
+      </c>
+      <c r="F4" t="s">
         <v>100</v>
-      </c>
-      <c r="D4" t="s">
-        <v>101</v>
-      </c>
-      <c r="E4" t="s">
-        <v>102</v>
-      </c>
-      <c r="F4" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="5">
@@ -1530,116 +1501,116 @@
         <v>47</v>
       </c>
       <c r="C5" t="s">
+        <v>101</v>
+      </c>
+      <c r="D5" t="s">
+        <v>102</v>
+      </c>
+      <c r="E5" t="s">
+        <v>103</v>
+      </c>
+      <c r="F5" t="s">
         <v>104</v>
-      </c>
-      <c r="D5" t="s">
-        <v>105</v>
-      </c>
-      <c r="E5" t="s">
-        <v>106</v>
-      </c>
-      <c r="F5" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B6" t="s">
         <v>55</v>
       </c>
       <c r="C6" t="s">
+        <v>106</v>
+      </c>
+      <c r="D6" t="s">
+        <v>107</v>
+      </c>
+      <c r="E6" t="s">
+        <v>108</v>
+      </c>
+      <c r="F6" t="s">
         <v>109</v>
-      </c>
-      <c r="D6" t="s">
-        <v>110</v>
-      </c>
-      <c r="E6" t="s">
-        <v>111</v>
-      </c>
-      <c r="F6" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B7" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D7" t="s">
+        <v>111</v>
+      </c>
+      <c r="E7" t="s">
+        <v>112</v>
+      </c>
+      <c r="F7" t="s">
         <v>113</v>
-      </c>
-      <c r="D7" t="s">
-        <v>114</v>
-      </c>
-      <c r="E7" t="s">
-        <v>115</v>
-      </c>
-      <c r="F7" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
+        <v>114</v>
+      </c>
+      <c r="B8" t="s">
+        <v>70</v>
+      </c>
+      <c r="C8" t="s">
+        <v>115</v>
+      </c>
+      <c r="D8" t="s">
+        <v>116</v>
+      </c>
+      <c r="E8" t="s">
         <v>117</v>
       </c>
-      <c r="B8" t="s">
-        <v>72</v>
-      </c>
-      <c r="C8" t="s">
+      <c r="F8" t="s">
         <v>118</v>
-      </c>
-      <c r="D8" t="s">
-        <v>119</v>
-      </c>
-      <c r="E8" t="s">
-        <v>120</v>
-      </c>
-      <c r="F8" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B9" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C9" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="D9" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E9" t="s">
+        <v>117</v>
+      </c>
+      <c r="F9" t="s">
         <v>120</v>
-      </c>
-      <c r="F9" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B10" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C10" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D10" t="s">
+        <v>119</v>
+      </c>
+      <c r="E10" t="s">
+        <v>117</v>
+      </c>
+      <c r="F10" t="s">
         <v>122</v>
-      </c>
-      <c r="E10" t="s">
-        <v>120</v>
-      </c>
-      <c r="F10" t="s">
-        <v>125</v>
       </c>
     </row>
   </sheetData>
@@ -1663,62 +1634,62 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="D1" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="E1" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="F1" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C2" t="s">
+        <v>128</v>
+      </c>
+      <c r="D2" t="s">
         <v>129</v>
       </c>
-      <c r="B2" t="s">
+      <c r="E2" t="s">
         <v>130</v>
       </c>
-      <c r="C2" t="s">
+      <c r="F2" t="s">
         <v>131</v>
-      </c>
-      <c r="D2" t="s">
-        <v>132</v>
-      </c>
-      <c r="E2" t="s">
-        <v>133</v>
-      </c>
-      <c r="F2" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
+        <v>132</v>
+      </c>
+      <c r="B3" t="s">
+        <v>133</v>
+      </c>
+      <c r="C3" t="s">
+        <v>128</v>
+      </c>
+      <c r="D3" t="s">
+        <v>129</v>
+      </c>
+      <c r="E3" t="s">
+        <v>134</v>
+      </c>
+      <c r="F3" t="s">
         <v>135</v>
-      </c>
-      <c r="B3" t="s">
-        <v>136</v>
-      </c>
-      <c r="C3" t="s">
-        <v>131</v>
-      </c>
-      <c r="D3" t="s">
-        <v>132</v>
-      </c>
-      <c r="E3" t="s">
-        <v>137</v>
-      </c>
-      <c r="F3" t="s">
-        <v>138</v>
       </c>
     </row>
   </sheetData>
@@ -1740,16 +1711,16 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B1" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="C1" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="D1" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="2">
@@ -1760,10 +1731,10 @@
         <v>2</v>
       </c>
       <c r="C2" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="D2" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
     <row r="3">
@@ -1774,7 +1745,7 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="D3" t="s">
         <v>18</v>
@@ -1788,24 +1759,24 @@
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="D4" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="B5" t="n">
         <v>1</v>
       </c>
       <c r="C5" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="D5" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
     <row r="6">
@@ -1813,13 +1784,13 @@
         <v>42</v>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C6" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="D6" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
     </row>
     <row r="7">
@@ -1830,38 +1801,38 @@
         <v>3</v>
       </c>
       <c r="C7" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="D7" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C8" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="D8" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B9" t="n">
         <v>6</v>
       </c>
       <c r="C9" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="D9" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
     </row>
   </sheetData>
@@ -1883,128 +1854,128 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="B1" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="C1" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="D1" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
+        <v>157</v>
+      </c>
+      <c r="B2" t="s">
+        <v>158</v>
+      </c>
+      <c r="C2" t="s">
+        <v>159</v>
+      </c>
+      <c r="D2" t="s">
         <v>160</v>
-      </c>
-      <c r="B2" t="s">
-        <v>161</v>
-      </c>
-      <c r="C2" t="s">
-        <v>162</v>
-      </c>
-      <c r="D2" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
+        <v>161</v>
+      </c>
+      <c r="B3" t="s">
+        <v>162</v>
+      </c>
+      <c r="C3" t="s">
+        <v>163</v>
+      </c>
+      <c r="D3" t="s">
         <v>164</v>
-      </c>
-      <c r="B3" t="s">
-        <v>165</v>
-      </c>
-      <c r="C3" t="s">
-        <v>166</v>
-      </c>
-      <c r="D3" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
+        <v>165</v>
+      </c>
+      <c r="B4" t="s">
+        <v>166</v>
+      </c>
+      <c r="C4" t="s">
+        <v>167</v>
+      </c>
+      <c r="D4" t="s">
         <v>168</v>
-      </c>
-      <c r="B4" t="s">
-        <v>169</v>
-      </c>
-      <c r="C4" t="s">
-        <v>170</v>
-      </c>
-      <c r="D4" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="B5" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="C5" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="D5" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
+        <v>172</v>
+      </c>
+      <c r="B6" t="s">
+        <v>173</v>
+      </c>
+      <c r="C6" t="s">
+        <v>174</v>
+      </c>
+      <c r="D6" t="s">
         <v>175</v>
-      </c>
-      <c r="B6" t="s">
-        <v>176</v>
-      </c>
-      <c r="C6" t="s">
-        <v>177</v>
-      </c>
-      <c r="D6" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="B7" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="C7" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="D7" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="B8" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="C8" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="D8" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
+        <v>182</v>
+      </c>
+      <c r="B9" t="s">
+        <v>183</v>
+      </c>
+      <c r="C9" t="s">
+        <v>184</v>
+      </c>
+      <c r="D9" t="s">
         <v>185</v>
-      </c>
-      <c r="B9" t="s">
-        <v>186</v>
-      </c>
-      <c r="C9" t="s">
-        <v>187</v>
-      </c>
-      <c r="D9" t="s">
-        <v>188</v>
       </c>
     </row>
   </sheetData>
@@ -2028,22 +1999,22 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B1" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="C1" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="D1" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="E1" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="F1" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="2">
@@ -2051,19 +2022,19 @@
         <v>12</v>
       </c>
       <c r="B2" t="s">
+        <v>189</v>
+      </c>
+      <c r="C2" t="s">
+        <v>190</v>
+      </c>
+      <c r="D2" t="s">
+        <v>191</v>
+      </c>
+      <c r="E2" t="s">
         <v>192</v>
       </c>
-      <c r="C2" t="s">
+      <c r="F2" t="s">
         <v>193</v>
-      </c>
-      <c r="D2" t="s">
-        <v>194</v>
-      </c>
-      <c r="E2" t="s">
-        <v>195</v>
-      </c>
-      <c r="F2" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="3">
@@ -2071,19 +2042,19 @@
         <v>23</v>
       </c>
       <c r="B3" t="s">
+        <v>194</v>
+      </c>
+      <c r="C3" t="s">
+        <v>195</v>
+      </c>
+      <c r="D3" t="s">
+        <v>196</v>
+      </c>
+      <c r="E3" t="s">
         <v>197</v>
       </c>
-      <c r="C3" t="s">
+      <c r="F3" t="s">
         <v>198</v>
-      </c>
-      <c r="D3" t="s">
-        <v>199</v>
-      </c>
-      <c r="E3" t="s">
-        <v>200</v>
-      </c>
-      <c r="F3" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="4">
@@ -2091,39 +2062,39 @@
         <v>27</v>
       </c>
       <c r="B4" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="C4" t="s">
+        <v>199</v>
+      </c>
+      <c r="D4" t="s">
+        <v>200</v>
+      </c>
+      <c r="E4" t="s">
+        <v>201</v>
+      </c>
+      <c r="F4" t="s">
         <v>202</v>
-      </c>
-      <c r="D4" t="s">
-        <v>203</v>
-      </c>
-      <c r="E4" t="s">
-        <v>204</v>
-      </c>
-      <c r="F4" t="s">
-        <v>205</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="B5" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="C5" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="D5" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="E5" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="F5" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
     </row>
     <row r="6">
@@ -2131,39 +2102,39 @@
         <v>42</v>
       </c>
       <c r="B6" t="s">
-        <v>192</v>
+        <v>205</v>
       </c>
       <c r="C6" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="D6" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="E6" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="F6" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
+        <v>207</v>
+      </c>
+      <c r="B7" t="s">
+        <v>208</v>
+      </c>
+      <c r="C7" t="s">
+        <v>197</v>
+      </c>
+      <c r="D7" t="s">
         <v>209</v>
       </c>
-      <c r="B7" t="s">
+      <c r="E7" t="s">
         <v>210</v>
       </c>
-      <c r="C7" t="s">
-        <v>200</v>
-      </c>
-      <c r="D7" t="s">
+      <c r="F7" t="s">
         <v>211</v>
-      </c>
-      <c r="E7" t="s">
-        <v>212</v>
-      </c>
-      <c r="F7" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="8">
@@ -2171,59 +2142,59 @@
         <v>51</v>
       </c>
       <c r="B8" t="s">
-        <v>214</v>
+        <v>205</v>
       </c>
       <c r="C8" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="D8" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="E8" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="F8" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B9" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C9" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="D9" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="E9" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="F9" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B10" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="C10" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="D10" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="E10" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="F10" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Zagreb just for Plitvice, extra day to Dubrovnik (4 nights)
</commit_message>
<xml_diff>
--- a/europe_nyc_trip_plan.xlsx
+++ b/europe_nyc_trip_plan.xlsx
@@ -145,328 +145,328 @@
     <t xml:space="preserve">Jun 2</t>
   </si>
   <si>
+    <t xml:space="preserve">Plitvice Lakes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Full day trip to Plitvice Lakes (bus 2-2.5h each way)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jun 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zagreb &gt; Dubrovnik</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Morning fly Zagreb &gt; Dubrovnik (Croatia Airlines)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jun 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dubrovnik</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Old Town, city walls walk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jun 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lokrum island, beaches</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jun 6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Elafiti islands day trip or Cavtat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jun 7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dubrovnik &gt; London</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fly Dubrovnik &gt; London Gatwick (easyJet)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jun 7-12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sun-Fri</t>
+  </si>
+  <si>
+    <t xml:space="preserve">London</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Free accommodation, explore London</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes (x6)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jun 13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">London &gt; LAX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fly London &gt; LAX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jun 13-18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sat-Thu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Home (LA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rest, possible dr's appt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jun 19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LAX &gt; NYC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evening fly LAX &gt; NYC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jun 19-25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NYC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NYC exploring, 1 room 1 bed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jun 26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JFK &gt; LAX (Person A)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Person A flies home</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jun 27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BWI &gt; LAX (Person B)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Person B flies home after wedding</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flight</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Airline</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Duration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Est_Price_PP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LAX &gt; Florence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">May 24-25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TBD (connection via Rome/Paris/London)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~14-16h total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$400-700</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arrive May 26 morning. Nonstop to Rome then connect, or via Paris/London</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ITA Airways (via Rome FCO)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~4-5h (1 stop)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$70-200</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ITA via FCO best option. No direct FLR-ATH on Thursdays</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aegean / Croatia Airlines / Ryanair</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~2-3h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$80-200</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Afternoon flight after ferry arrives ~noon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Croatia Airlines / Eurowings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~1h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$50-120</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Short morning hop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dubrovnik &gt; London Gatwick</t>
+  </si>
+  <si>
+    <t xml:space="preserve">easyJet (direct)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~2.5h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$40-100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Direct to Gatwick, ~2.5h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TBD (direct or 1-stop)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~11h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$300-500</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Direct options: BA, Virgin, AA, United, Norse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LAX &gt; NYC (JFK)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JetBlue / Delta / AA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~5h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$100-250</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evening departure after dr's appt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~5.5h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Person A returns home</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Southwest / AA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Person B returns after wedding</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Route</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Operator</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Est_Cost_PP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Piraeus &gt; Paros</t>
+  </si>
+  <si>
+    <t xml:space="preserve">May 29 (Fri)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.5-4.5h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blue Star / SeaJets / Hellenic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$45-80</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Morning departure from Piraeus Gate E7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paros &gt; Piraeus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">May 31 (Sun)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$45-70</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Early morning departure, arrive Piraeus by noon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">City</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nights</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Est_Cost_Per_Night</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$120-180</t>
+  </si>
+  <si>
+    <t xml:space="preserve">May 26-27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$80-120</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$90-150</t>
+  </si>
+  <si>
+    <t xml:space="preserve">May 29-30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Athens (return)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">May 31 (after ferry)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Zagreb</t>
   </si>
   <si>
-    <t xml:space="preserve">Explore Zagreb Upper Town, Dolac Market, food scene</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jun 3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Plitvice Lakes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Full day trip to Plitvice Lakes (bus 2-2.5h each way)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jun 4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zagreb &gt; Dubrovnik</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Morning fly Zagreb &gt; Dubrovnik (Croatia Airlines)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jun 5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dubrovnik</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Old Town, city walls walk</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jun 6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lokrum island, beaches</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jun 7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dubrovnik &gt; London</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fly Dubrovnik &gt; London Gatwick (easyJet)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jun 7-12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sun-Fri</t>
-  </si>
-  <si>
-    <t xml:space="preserve">London</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Free accommodation, explore London</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yes (x6)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jun 13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">London &gt; LAX</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fly London &gt; LAX</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jun 13-18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sat-Thu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Home (LA)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rest, possible dr's appt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jun 19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LAX &gt; NYC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Evening fly LAX &gt; NYC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jun 19-25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NYC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NYC exploring, 1 room 1 bed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jun 26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JFK &gt; LAX (Person A)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Person A flies home</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jun 27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BWI &gt; LAX (Person B)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Person B flies home after wedding</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Flight</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Airline</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Duration</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Est_Price_PP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Notes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LAX &gt; Florence</t>
-  </si>
-  <si>
-    <t xml:space="preserve">May 24-25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TBD (connection via Rome/Paris/London)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">~14-16h total</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$400-700</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Arrive May 26 morning. Nonstop to Rome then connect, or via Paris/London</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ITA Airways (via Rome FCO)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">~4-5h (1 stop)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$70-200</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ITA via FCO best option. No direct FLR-ATH on Thursdays</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aegean / Croatia Airlines / Ryanair</t>
-  </si>
-  <si>
-    <t xml:space="preserve">~2-3h</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$80-200</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Afternoon flight after ferry arrives ~noon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Croatia Airlines / Eurowings</t>
-  </si>
-  <si>
-    <t xml:space="preserve">~1h</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$50-120</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Short morning hop</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dubrovnik &gt; London Gatwick</t>
-  </si>
-  <si>
-    <t xml:space="preserve">easyJet (direct)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">~2.5h</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$40-100</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Direct to Gatwick, ~2.5h</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TBD (direct or 1-stop)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">~11h</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$300-500</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Direct options: BA, Virgin, AA, United, Norse</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LAX &gt; NYC (JFK)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JetBlue / Delta / AA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">~5h</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$100-250</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Evening departure after dr's appt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">~5.5h</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Person A returns home</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Southwest / AA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Person B returns after wedding</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Route</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Operator</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Est_Cost_PP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Piraeus &gt; Paros</t>
-  </si>
-  <si>
-    <t xml:space="preserve">May 29 (Fri)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.5-4.5h</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Blue Star / SeaJets / Hellenic</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$45-80</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Morning departure from Piraeus Gate E7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Paros &gt; Piraeus</t>
-  </si>
-  <si>
-    <t xml:space="preserve">May 31 (Sun)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$45-70</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Early morning departure, arrive Piraeus by noon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">City</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nights</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Est_Cost_Per_Night</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$120-180</t>
-  </si>
-  <si>
-    <t xml:space="preserve">May 26-27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$80-120</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$90-150</t>
-  </si>
-  <si>
-    <t xml:space="preserve">May 29-30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Athens (return)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">May 31 (after ferry)</t>
-  </si>
-  <si>
     <t xml:space="preserve">$60-100</t>
   </si>
   <si>
-    <t xml:space="preserve">Jun 1-3 (arrive Mon evening)</t>
+    <t xml:space="preserve">Jun 1-2 (Plitvice day trip Jun 2)</t>
   </si>
   <si>
     <t xml:space="preserve">$80-140</t>
   </si>
   <si>
-    <t xml:space="preserve">Jun 4-6</t>
+    <t xml:space="preserve">Jun 3-6</t>
   </si>
   <si>
     <t xml:space="preserve">Free</t>
@@ -523,7 +523,7 @@
     <t xml:space="preserve">$3,300</t>
   </si>
   <si>
-    <t xml:space="preserve">2 Florence + 1 Athens + 2 Paros + 1 Athens return + 3 Zagreb + 3 Dubrovnik + 6 NYC</t>
+    <t xml:space="preserve">2 Florence + 1 Athens + 2 Paros + 1 Athens return + 2 Zagreb + 4 Dubrovnik + 6 NYC</t>
   </si>
   <si>
     <t xml:space="preserve">Food &amp; Drink</t>
@@ -634,10 +634,7 @@
     <t xml:space="preserve">Overnight before Zagreb flight</t>
   </si>
   <si>
-    <t xml:space="preserve">3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Upper Town, Dolac Market, food scene</t>
+    <t xml:space="preserve">Plitvice day trip base</t>
   </si>
   <si>
     <t xml:space="preserve">Plitvice entrance</t>
@@ -653,6 +650,9 @@
   </si>
   <si>
     <t xml:space="preserve">Park entrance ~$25/pp, bus ~$15-18/pp each way</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4</t>
   </si>
   <si>
     <t xml:space="preserve">$15-30</t>
@@ -1204,7 +1204,7 @@
         <v>46</v>
       </c>
       <c r="E12" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13">
@@ -1232,10 +1232,10 @@
         <v>26</v>
       </c>
       <c r="C14" t="s">
+        <v>48</v>
+      </c>
+      <c r="D14" t="s">
         <v>51</v>
-      </c>
-      <c r="D14" t="s">
-        <v>52</v>
       </c>
       <c r="E14" t="s">
         <v>14</v>
@@ -1243,16 +1243,16 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B15" t="s">
         <v>30</v>
       </c>
       <c r="C15" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D15" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E15" t="s">
         <v>14</v>
@@ -1260,16 +1260,16 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B16" t="s">
         <v>33</v>
       </c>
       <c r="C16" t="s">
+        <v>55</v>
+      </c>
+      <c r="D16" t="s">
         <v>56</v>
-      </c>
-      <c r="D16" t="s">
-        <v>57</v>
       </c>
       <c r="E16" t="s">
         <v>9</v>
@@ -1277,33 +1277,33 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
+        <v>57</v>
+      </c>
+      <c r="B17" t="s">
         <v>58</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C17" t="s">
         <v>59</v>
       </c>
-      <c r="C17" t="s">
+      <c r="D17" t="s">
         <v>60</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" t="s">
         <v>61</v>
-      </c>
-      <c r="E17" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B18" t="s">
         <v>30</v>
       </c>
       <c r="C18" t="s">
+        <v>63</v>
+      </c>
+      <c r="D18" t="s">
         <v>64</v>
-      </c>
-      <c r="D18" t="s">
-        <v>65</v>
       </c>
       <c r="E18" t="s">
         <v>9</v>
@@ -1311,16 +1311,16 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
+        <v>65</v>
+      </c>
+      <c r="B19" t="s">
         <v>66</v>
       </c>
-      <c r="B19" t="s">
+      <c r="C19" t="s">
         <v>67</v>
       </c>
-      <c r="C19" t="s">
+      <c r="D19" t="s">
         <v>68</v>
-      </c>
-      <c r="D19" t="s">
-        <v>69</v>
       </c>
       <c r="E19" t="s">
         <v>9</v>
@@ -1328,16 +1328,16 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B20" t="s">
         <v>26</v>
       </c>
       <c r="C20" t="s">
+        <v>70</v>
+      </c>
+      <c r="D20" t="s">
         <v>71</v>
-      </c>
-      <c r="D20" t="s">
-        <v>72</v>
       </c>
       <c r="E20" t="s">
         <v>9</v>
@@ -1345,33 +1345,33 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
+        <v>72</v>
+      </c>
+      <c r="B21" t="s">
+        <v>66</v>
+      </c>
+      <c r="C21" t="s">
         <v>73</v>
       </c>
-      <c r="B21" t="s">
-        <v>67</v>
-      </c>
-      <c r="C21" t="s">
+      <c r="D21" t="s">
         <v>74</v>
       </c>
-      <c r="D21" t="s">
-        <v>75</v>
-      </c>
       <c r="E21" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B22" t="s">
         <v>26</v>
       </c>
       <c r="C22" t="s">
+        <v>76</v>
+      </c>
+      <c r="D22" t="s">
         <v>77</v>
-      </c>
-      <c r="D22" t="s">
-        <v>78</v>
       </c>
       <c r="E22" t="s">
         <v>9</v>
@@ -1379,16 +1379,16 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B23" t="s">
         <v>30</v>
       </c>
       <c r="C23" t="s">
+        <v>79</v>
+      </c>
+      <c r="D23" t="s">
         <v>80</v>
-      </c>
-      <c r="D23" t="s">
-        <v>81</v>
       </c>
       <c r="E23" t="s">
         <v>9</v>
@@ -1415,42 +1415,42 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
       </c>
       <c r="C1" t="s">
+        <v>82</v>
+      </c>
+      <c r="D1" t="s">
         <v>83</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>84</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>85</v>
-      </c>
-      <c r="F1" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B2" t="s">
         <v>87</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>88</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>89</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>90</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>91</v>
-      </c>
-      <c r="F2" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="3">
@@ -1461,16 +1461,16 @@
         <v>18</v>
       </c>
       <c r="C3" t="s">
+        <v>92</v>
+      </c>
+      <c r="D3" t="s">
         <v>93</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>94</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>95</v>
-      </c>
-      <c r="F3" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="4">
@@ -1481,136 +1481,136 @@
         <v>41</v>
       </c>
       <c r="C4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D4" t="s">
         <v>97</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>98</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>99</v>
-      </c>
-      <c r="F4" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B5" t="s">
         <v>47</v>
       </c>
       <c r="C5" t="s">
+        <v>100</v>
+      </c>
+      <c r="D5" t="s">
         <v>101</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>102</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>103</v>
-      </c>
-      <c r="F5" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
+        <v>104</v>
+      </c>
+      <c r="B6" t="s">
+        <v>54</v>
+      </c>
+      <c r="C6" t="s">
         <v>105</v>
       </c>
-      <c r="B6" t="s">
-        <v>55</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>106</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>107</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>108</v>
-      </c>
-      <c r="F6" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B7" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C7" t="s">
+        <v>109</v>
+      </c>
+      <c r="D7" t="s">
         <v>110</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>111</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>112</v>
-      </c>
-      <c r="F7" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
+        <v>113</v>
+      </c>
+      <c r="B8" t="s">
+        <v>69</v>
+      </c>
+      <c r="C8" t="s">
         <v>114</v>
       </c>
-      <c r="B8" t="s">
-        <v>70</v>
-      </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>115</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>116</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
         <v>117</v>
-      </c>
-      <c r="F8" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C9" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D9" t="s">
+        <v>118</v>
+      </c>
+      <c r="E9" t="s">
+        <v>116</v>
+      </c>
+      <c r="F9" t="s">
         <v>119</v>
-      </c>
-      <c r="E9" t="s">
-        <v>117</v>
-      </c>
-      <c r="F9" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B10" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C10" t="s">
+        <v>120</v>
+      </c>
+      <c r="D10" t="s">
+        <v>118</v>
+      </c>
+      <c r="E10" t="s">
+        <v>116</v>
+      </c>
+      <c r="F10" t="s">
         <v>121</v>
-      </c>
-      <c r="D10" t="s">
-        <v>119</v>
-      </c>
-      <c r="E10" t="s">
-        <v>117</v>
-      </c>
-      <c r="F10" t="s">
-        <v>122</v>
       </c>
     </row>
   </sheetData>
@@ -1634,62 +1634,62 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D1" t="s">
+        <v>123</v>
+      </c>
+      <c r="E1" t="s">
         <v>124</v>
       </c>
-      <c r="E1" t="s">
-        <v>125</v>
-      </c>
       <c r="F1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B2" t="s">
         <v>126</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>127</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>128</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>129</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>130</v>
-      </c>
-      <c r="F2" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
+        <v>131</v>
+      </c>
+      <c r="B3" t="s">
         <v>132</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
+        <v>127</v>
+      </c>
+      <c r="D3" t="s">
+        <v>128</v>
+      </c>
+      <c r="E3" t="s">
         <v>133</v>
       </c>
-      <c r="C3" t="s">
-        <v>128</v>
-      </c>
-      <c r="D3" t="s">
-        <v>129</v>
-      </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>134</v>
-      </c>
-      <c r="F3" t="s">
-        <v>135</v>
       </c>
     </row>
   </sheetData>
@@ -1706,21 +1706,21 @@
     <col min="1" max="1" width="15.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="6.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="18.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="32.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="33.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
+        <v>135</v>
+      </c>
+      <c r="B1" t="s">
         <v>136</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>137</v>
       </c>
-      <c r="C1" t="s">
-        <v>138</v>
-      </c>
       <c r="D1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="2">
@@ -1731,10 +1731,10 @@
         <v>2</v>
       </c>
       <c r="C2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D2" t="s">
         <v>139</v>
-      </c>
-      <c r="D2" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="3">
@@ -1745,7 +1745,7 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D3" t="s">
         <v>18</v>
@@ -1759,32 +1759,32 @@
         <v>2</v>
       </c>
       <c r="C4" t="s">
+        <v>141</v>
+      </c>
+      <c r="D4" t="s">
         <v>142</v>
-      </c>
-      <c r="D4" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B5" t="n">
         <v>1</v>
       </c>
       <c r="C5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>42</v>
+        <v>145</v>
       </c>
       <c r="B6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C6" t="s">
         <v>146</v>
@@ -1795,10 +1795,10 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C7" t="s">
         <v>148</v>
@@ -1809,7 +1809,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B8" t="n">
         <v>6</v>
@@ -1823,7 +1823,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B9" t="n">
         <v>6</v>
@@ -1863,7 +1863,7 @@
         <v>156</v>
       </c>
       <c r="D1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="2">
@@ -1999,10 +1999,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
+        <v>135</v>
+      </c>
+      <c r="B1" t="s">
         <v>136</v>
-      </c>
-      <c r="B1" t="s">
-        <v>137</v>
       </c>
       <c r="C1" t="s">
         <v>186</v>
@@ -2014,7 +2014,7 @@
         <v>188</v>
       </c>
       <c r="F1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="2">
@@ -2079,7 +2079,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B5" t="s">
         <v>194</v>
@@ -2099,10 +2099,10 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>42</v>
+        <v>145</v>
       </c>
       <c r="B6" t="s">
-        <v>205</v>
+        <v>189</v>
       </c>
       <c r="C6" t="s">
         <v>195</v>
@@ -2114,35 +2114,35 @@
         <v>200</v>
       </c>
       <c r="F6" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
+        <v>206</v>
+      </c>
+      <c r="B7" t="s">
         <v>207</v>
-      </c>
-      <c r="B7" t="s">
-        <v>208</v>
       </c>
       <c r="C7" t="s">
         <v>197</v>
       </c>
       <c r="D7" t="s">
+        <v>208</v>
+      </c>
+      <c r="E7" t="s">
         <v>209</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>210</v>
-      </c>
-      <c r="F7" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B8" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="C8" t="s">
         <v>199</v>
@@ -2159,7 +2159,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B9" t="s">
         <v>214</v>
@@ -2179,7 +2179,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B10" t="s">
         <v>214</v>

</xml_diff>

<commit_message>
Add Montenegro day trip from Dubrovnik
</commit_message>
<xml_diff>
--- a/europe_nyc_trip_plan.xlsx
+++ b/europe_nyc_trip_plan.xlsx
@@ -157,7 +157,7 @@
     <t xml:space="preserve">Zagreb &gt; Dubrovnik</t>
   </si>
   <si>
-    <t xml:space="preserve">Morning fly Zagreb &gt; Dubrovnik (Croatia Airlines)</t>
+    <t xml:space="preserve">Morning fly Zagreb &gt; Dubrovnik, settle in, evening Old Town stroll</t>
   </si>
   <si>
     <t xml:space="preserve">Jun 4</t>
@@ -166,19 +166,19 @@
     <t xml:space="preserve">Dubrovnik</t>
   </si>
   <si>
-    <t xml:space="preserve">Old Town, city walls walk</t>
+    <t xml:space="preserve">Day trip to Montenegro: Bay of Kotor, Perast, Kotor Old Town</t>
   </si>
   <si>
     <t xml:space="preserve">Jun 5</t>
   </si>
   <si>
-    <t xml:space="preserve">Lokrum island, beaches</t>
+    <t xml:space="preserve">City walls walk, Lokrum island</t>
   </si>
   <si>
     <t xml:space="preserve">Jun 6</t>
   </si>
   <si>
-    <t xml:space="preserve">Elafiti islands day trip or Cavtat</t>
+    <t xml:space="preserve">Beach day, Old Town exploring, sunset drinks</t>
   </si>
   <si>
     <t xml:space="preserve">Jun 7</t>
@@ -999,7 +999,7 @@
     <col min="1" max="1" width="9.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="7.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="23.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="59.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="69.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="16.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1204,7 +1204,7 @@
         <v>46</v>
       </c>
       <c r="E12" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
Montenegro day trip: self-guided bus to Kotor
</commit_message>
<xml_diff>
--- a/europe_nyc_trip_plan.xlsx
+++ b/europe_nyc_trip_plan.xlsx
@@ -166,7 +166,7 @@
     <t xml:space="preserve">Dubrovnik</t>
   </si>
   <si>
-    <t xml:space="preserve">Day trip to Montenegro: Bay of Kotor, Perast, Kotor Old Town</t>
+    <t xml:space="preserve">Bus to Kotor (~2h, ~$30/pp), Old Town, fortress hike, Perast + Our Lady of the Rocks, bus back</t>
   </si>
   <si>
     <t xml:space="preserve">Jun 5</t>
@@ -999,7 +999,7 @@
     <col min="1" max="1" width="9.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="7.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="23.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="69.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="94.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="16.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>

<commit_message>
London +1 night (leave Jun 14), NYC depart Jun 18 evening
</commit_message>
<xml_diff>
--- a/europe_nyc_trip_plan.xlsx
+++ b/europe_nyc_trip_plan.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="221">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -157,7 +157,7 @@
     <t xml:space="preserve">Zagreb &gt; Dubrovnik</t>
   </si>
   <si>
-    <t xml:space="preserve">Morning fly Zagreb &gt; Dubrovnik, settle in, evening Old Town stroll</t>
+    <t xml:space="preserve">Morning fly Zagreb &gt; Dubrovnik (Croatia Airlines)</t>
   </si>
   <si>
     <t xml:space="preserve">Jun 4</t>
@@ -172,13 +172,13 @@
     <t xml:space="preserve">Jun 5</t>
   </si>
   <si>
-    <t xml:space="preserve">City walls walk, Lokrum island</t>
+    <t xml:space="preserve">Old Town, city walls walk, Lokrum island</t>
   </si>
   <si>
     <t xml:space="preserve">Jun 6</t>
   </si>
   <si>
-    <t xml:space="preserve">Beach day, Old Town exploring, sunset drinks</t>
+    <t xml:space="preserve">Beach day, exploring, sunset drinks</t>
   </si>
   <si>
     <t xml:space="preserve">Jun 7</t>
@@ -190,10 +190,10 @@
     <t xml:space="preserve">Fly Dubrovnik &gt; London Gatwick (easyJet)</t>
   </si>
   <si>
-    <t xml:space="preserve">Jun 7-12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sun-Fri</t>
+    <t xml:space="preserve">Jun 7-13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sun-Sat</t>
   </si>
   <si>
     <t xml:space="preserve">London</t>
@@ -202,165 +202,174 @@
     <t xml:space="preserve">Free accommodation, explore London</t>
   </si>
   <si>
-    <t xml:space="preserve">Yes (x6)</t>
+    <t xml:space="preserve">Yes (x7)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jun 14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">London &gt; LAX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fly London &gt; LAX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jun 14-17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sun-Wed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Home (LA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rest, possible dr's appt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jun 18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LAX &gt; NYC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evening fly LAX &gt; NYC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jun 18-25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thu-Thu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NYC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NYC exploring, 1 room 1 bed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jun 26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JFK &gt; LAX (Person A)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Person A flies home</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jun 27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BWI &gt; LAX (Person B)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Person B flies home after wedding</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flight</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Airline</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Duration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Est_Price_PP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LAX &gt; Florence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">May 24-25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TBD (connection via Rome/Paris/London)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~14-16h total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$400-700</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arrive May 26 morning. Nonstop to Rome then connect, or via Paris/London</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ITA Airways (via Rome FCO)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~4-5h (1 stop)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$70-200</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ITA via FCO best option. No direct FLR-ATH on Thursdays</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aegean / Croatia Airlines / Ryanair</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~2-3h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$80-200</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Afternoon flight after ferry arrives ~noon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Croatia Airlines / Eurowings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~1h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$50-120</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Short morning hop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dubrovnik &gt; London Gatwick</t>
+  </si>
+  <si>
+    <t xml:space="preserve">easyJet (direct)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~2.5h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$40-100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Direct to Gatwick, ~2.5h</t>
   </si>
   <si>
     <t xml:space="preserve">Jun 13</t>
   </si>
   <si>
-    <t xml:space="preserve">London &gt; LAX</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fly London &gt; LAX</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jun 13-18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sat-Thu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Home (LA)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rest, possible dr's appt</t>
+    <t xml:space="preserve">TBD (direct or 1-stop)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~11h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$300-500</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Direct options: BA, Virgin, AA, United, Norse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LAX &gt; NYC (JFK)</t>
   </si>
   <si>
     <t xml:space="preserve">Jun 19</t>
   </si>
   <si>
-    <t xml:space="preserve">LAX &gt; NYC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Evening fly LAX &gt; NYC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jun 19-25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NYC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NYC exploring, 1 room 1 bed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jun 26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">JFK &gt; LAX (Person A)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Person A flies home</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jun 27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BWI &gt; LAX (Person B)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Person B flies home after wedding</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Flight</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Airline</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Duration</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Est_Price_PP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Notes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LAX &gt; Florence</t>
-  </si>
-  <si>
-    <t xml:space="preserve">May 24-25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TBD (connection via Rome/Paris/London)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">~14-16h total</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$400-700</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Arrive May 26 morning. Nonstop to Rome then connect, or via Paris/London</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ITA Airways (via Rome FCO)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">~4-5h (1 stop)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$70-200</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ITA via FCO best option. No direct FLR-ATH on Thursdays</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aegean / Croatia Airlines / Ryanair</t>
-  </si>
-  <si>
-    <t xml:space="preserve">~2-3h</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$80-200</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Afternoon flight after ferry arrives ~noon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Croatia Airlines / Eurowings</t>
-  </si>
-  <si>
-    <t xml:space="preserve">~1h</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$50-120</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Short morning hop</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dubrovnik &gt; London Gatwick</t>
-  </si>
-  <si>
-    <t xml:space="preserve">easyJet (direct)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">~2.5h</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$40-100</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Direct to Gatwick, ~2.5h</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TBD (direct or 1-stop)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">~11h</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$300-500</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Direct options: BA, Virgin, AA, United, Norse</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LAX &gt; NYC (JFK)</t>
-  </si>
-  <si>
     <t xml:space="preserve">JetBlue / Delta / AA</t>
   </si>
   <si>
@@ -460,7 +469,7 @@
     <t xml:space="preserve">$60-100</t>
   </si>
   <si>
-    <t xml:space="preserve">Jun 1-2 (Plitvice day trip Jun 2)</t>
+    <t xml:space="preserve">Jun 1-2</t>
   </si>
   <si>
     <t xml:space="preserve">$80-140</t>
@@ -472,13 +481,13 @@
     <t xml:space="preserve">Free</t>
   </si>
   <si>
-    <t xml:space="preserve">Jun 7-12 (free)</t>
+    <t xml:space="preserve">Jun 7-13 (free)</t>
   </si>
   <si>
     <t xml:space="preserve">$150-250</t>
   </si>
   <si>
-    <t xml:space="preserve">Jun 19-25 (1 room, 1 bed, 2 ppl)</t>
+    <t xml:space="preserve">Jun 18-25 (1 room, 1 bed, 2 ppl)</t>
   </si>
   <si>
     <t xml:space="preserve">Category</t>
@@ -514,25 +523,28 @@
     <t xml:space="preserve">2 ferries x 2 people</t>
   </si>
   <si>
-    <t xml:space="preserve">Accommodation (18 paid nights)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$1,860</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$3,300</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2 Florence + 1 Athens + 2 Paros + 1 Athens return + 2 Zagreb + 4 Dubrovnik + 6 NYC</t>
+    <t xml:space="preserve">Accommodation (19 paid nights)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$2,010</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$3,550</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 Florence + 1 Athens + 2 Paros + 1 Athens return + 2 Zagreb + 4 Dubrovnik + 7 NYC</t>
   </si>
   <si>
     <t xml:space="preserve">Food &amp; Drink</t>
   </si>
   <si>
-    <t xml:space="preserve">$1,400</t>
-  </si>
-  <si>
-    <t xml:space="preserve">~24 days of eating</t>
+    <t xml:space="preserve">$1,500</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$2,600</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~26 days of eating</t>
   </si>
   <si>
     <t xml:space="preserve">Activities &amp; Entrance Fees</t>
@@ -544,7 +556,7 @@
     <t xml:space="preserve">$800</t>
   </si>
   <si>
-    <t xml:space="preserve">Museums, Plitvice, kayak, cooking class, walls</t>
+    <t xml:space="preserve">Museums, Plitvice, kayak, cooking class, walls, Kotor bus</t>
   </si>
   <si>
     <t xml:space="preserve">Local Transport</t>
@@ -568,10 +580,10 @@
     <t xml:space="preserve">TOTAL (2 people)</t>
   </si>
   <si>
-    <t xml:space="preserve">$6,740</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$11,900</t>
+    <t xml:space="preserve">$6,990</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$12,350</t>
   </si>
   <si>
     <t xml:space="preserve">For 2 people total</t>
@@ -658,10 +670,10 @@
     <t xml:space="preserve">$15-30</t>
   </si>
   <si>
-    <t xml:space="preserve">Walls ticket ~$35, Lokrum ferry ~$15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6</t>
+    <t xml:space="preserve">Walls ticket ~$35, Lokrum ferry ~$15, Kotor bus ~$30/pp RT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7</t>
   </si>
   <si>
     <t xml:space="preserve">Free accommodation helps a lot</t>
@@ -1204,7 +1216,7 @@
         <v>46</v>
       </c>
       <c r="E12" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13">
@@ -1297,7 +1309,7 @@
         <v>62</v>
       </c>
       <c r="B18" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C18" t="s">
         <v>63</v>
@@ -1331,7 +1343,7 @@
         <v>69</v>
       </c>
       <c r="B20" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="C20" t="s">
         <v>70</v>
@@ -1348,13 +1360,13 @@
         <v>72</v>
       </c>
       <c r="B21" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="C21" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D21" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E21" t="s">
         <v>61</v>
@@ -1362,16 +1374,16 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B22" t="s">
         <v>26</v>
       </c>
       <c r="C22" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D22" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E22" t="s">
         <v>9</v>
@@ -1379,16 +1391,16 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B23" t="s">
         <v>30</v>
       </c>
       <c r="C23" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D23" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E23" t="s">
         <v>9</v>
@@ -1415,42 +1427,42 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="3">
@@ -1461,16 +1473,16 @@
         <v>18</v>
       </c>
       <c r="C3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="4">
@@ -1481,16 +1493,16 @@
         <v>41</v>
       </c>
       <c r="C4" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F4" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5">
@@ -1501,36 +1513,36 @@
         <v>47</v>
       </c>
       <c r="C5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B6" t="s">
         <v>54</v>
       </c>
       <c r="C6" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="7">
@@ -1538,79 +1550,79 @@
         <v>63</v>
       </c>
       <c r="B7" t="s">
-        <v>62</v>
+        <v>110</v>
       </c>
       <c r="C7" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D7" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E7" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F7" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B8" t="s">
-        <v>69</v>
+        <v>116</v>
       </c>
       <c r="C8" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="D8" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="E8" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="F8" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
+        <v>77</v>
+      </c>
+      <c r="B9" t="s">
         <v>76</v>
       </c>
-      <c r="B9" t="s">
-        <v>75</v>
-      </c>
       <c r="C9" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="D9" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="E9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="F9" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
+        <v>80</v>
+      </c>
+      <c r="B10" t="s">
         <v>79</v>
       </c>
-      <c r="B10" t="s">
-        <v>78</v>
-      </c>
       <c r="C10" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="D10" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="E10" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="F10" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -1634,62 +1646,62 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="E1" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="F1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B2" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="C2" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="D2" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="E2" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="F2" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
+        <v>134</v>
+      </c>
+      <c r="B3" t="s">
+        <v>135</v>
+      </c>
+      <c r="C3" t="s">
+        <v>130</v>
+      </c>
+      <c r="D3" t="s">
         <v>131</v>
       </c>
-      <c r="B3" t="s">
-        <v>132</v>
-      </c>
-      <c r="C3" t="s">
-        <v>127</v>
-      </c>
-      <c r="D3" t="s">
-        <v>128</v>
-      </c>
       <c r="E3" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="F3" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
     </row>
   </sheetData>
@@ -1706,21 +1718,21 @@
     <col min="1" max="1" width="15.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="6.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="18.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="33.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="32.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="B1" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="C1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="D1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="2">
@@ -1731,10 +1743,10 @@
         <v>2</v>
       </c>
       <c r="C2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="D2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
     </row>
     <row r="3">
@@ -1745,7 +1757,7 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="D3" t="s">
         <v>18</v>
@@ -1759,38 +1771,38 @@
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="D4" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B5" t="n">
         <v>1</v>
       </c>
       <c r="C5" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="D5" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="B6" t="n">
         <v>2</v>
       </c>
       <c r="C6" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="D6" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
     </row>
     <row r="7">
@@ -1801,10 +1813,10 @@
         <v>4</v>
       </c>
       <c r="C7" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="D7" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
     </row>
     <row r="8">
@@ -1812,27 +1824,27 @@
         <v>59</v>
       </c>
       <c r="B8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C8" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="D8" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C9" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="D9" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
     </row>
   </sheetData>
@@ -1854,128 +1866,128 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="B1" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="C1" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="D1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="B2" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="C2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="D2" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="B3" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="C3" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="D3" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="B4" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="C4" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="D4" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="B5" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="C5" t="s">
-        <v>158</v>
+        <v>174</v>
       </c>
       <c r="D5" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="B6" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="C6" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="D6" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="B7" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="C7" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="D7" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="B8" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="C8" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="D8" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="B9" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="C9" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="D9" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
     </row>
   </sheetData>
@@ -1994,27 +2006,27 @@
     <col min="3" max="3" width="12.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="17.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="18.71" hidden="0" customWidth="1"/>
-    <col min="6" max="6" width="46.71" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="58.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="B1" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="C1" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="D1" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="E1" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="F1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="2">
@@ -2022,19 +2034,19 @@
         <v>12</v>
       </c>
       <c r="B2" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="C2" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="D2" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="E2" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="F2" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
     </row>
     <row r="3">
@@ -2042,19 +2054,19 @@
         <v>23</v>
       </c>
       <c r="B3" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="C3" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="D3" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="E3" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="F3" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
     </row>
     <row r="4">
@@ -2062,79 +2074,79 @@
         <v>27</v>
       </c>
       <c r="B4" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="C4" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="D4" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="E4" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="F4" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B5" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="C5" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="D5" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="E5" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="F5" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="B6" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="C6" t="s">
+        <v>199</v>
+      </c>
+      <c r="D6" t="s">
         <v>195</v>
       </c>
-      <c r="D6" t="s">
-        <v>191</v>
-      </c>
       <c r="E6" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="F6" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="B7" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="C7" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="D7" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="E7" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="F7" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="8">
@@ -2142,19 +2154,19 @@
         <v>48</v>
       </c>
       <c r="B8" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="C8" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="D8" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="E8" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="F8" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
     </row>
     <row r="9">
@@ -2162,39 +2174,39 @@
         <v>59</v>
       </c>
       <c r="B9" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="C9" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="D9" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="E9" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="F9" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B10" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="C10" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="D10" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="E10" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="F10" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
NYC 6 nights (Jun 19-24), morning LAX>JFK, re-priced budget
Shift LAX>JFK from Jun 18 evening to Jun 19 morning, cutting
NYC to 6 nights. Re-priced flights and accommodation for
last-minute May 2026 booking; updated totals: $9,140 - $15,630.
</commit_message>
<xml_diff>
--- a/europe_nyc_trip_plan.xlsx
+++ b/europe_nyc_trip_plan.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="225">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -166,7 +166,7 @@
     <t xml:space="preserve">Dubrovnik</t>
   </si>
   <si>
-    <t xml:space="preserve">Bus to Kotor (~2h, ~$30/pp), Old Town, fortress hike, Perast + Our Lady of the Rocks, bus back</t>
+    <t xml:space="preserve">Bus to Kotor (~2h, ~$30/pp), Old Town, fortress hike, Perast + Our Lady of the Rocks</t>
   </si>
   <si>
     <t xml:space="preserve">Jun 5</t>
@@ -214,10 +214,10 @@
     <t xml:space="preserve">Fly London &gt; LAX</t>
   </si>
   <si>
-    <t xml:space="preserve">Jun 14-17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sun-Wed</t>
+    <t xml:space="preserve">Jun 14-18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sun-Thu</t>
   </si>
   <si>
     <t xml:space="preserve">Home (LA)</t>
@@ -226,19 +226,19 @@
     <t xml:space="preserve">Rest, possible dr's appt</t>
   </si>
   <si>
-    <t xml:space="preserve">Jun 18</t>
+    <t xml:space="preserve">Jun 19</t>
   </si>
   <si>
     <t xml:space="preserve">LAX &gt; NYC</t>
   </si>
   <si>
-    <t xml:space="preserve">Evening fly LAX &gt; NYC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jun 18-25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thu-Thu</t>
+    <t xml:space="preserve">Morning fly LAX &gt; NYC (arrive afternoon/evening)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jun 19-25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fri-Thu</t>
   </si>
   <si>
     <t xml:space="preserve">NYC</t>
@@ -247,6 +247,9 @@
     <t xml:space="preserve">NYC exploring, 1 room 1 bed</t>
   </si>
   <si>
+    <t xml:space="preserve">Yes (x6)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Jun 26</t>
   </si>
   <si>
@@ -292,10 +295,10 @@
     <t xml:space="preserve">~14-16h total</t>
   </si>
   <si>
-    <t xml:space="preserve">$400-700</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Arrive May 26 morning. Nonstop to Rome then connect, or via Paris/London</t>
+    <t xml:space="preserve">$700-1100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Last-minute booking; nonstop to Rome then connect, or via Paris/London</t>
   </si>
   <si>
     <t xml:space="preserve">ITA Airways (via Rome FCO)</t>
@@ -304,7 +307,7 @@
     <t xml:space="preserve">~4-5h (1 stop)</t>
   </si>
   <si>
-    <t xml:space="preserve">$70-200</t>
+    <t xml:space="preserve">$120-220</t>
   </si>
   <si>
     <t xml:space="preserve">ITA via FCO best option. No direct FLR-ATH on Thursdays</t>
@@ -316,7 +319,7 @@
     <t xml:space="preserve">~2-3h</t>
   </si>
   <si>
-    <t xml:space="preserve">$80-200</t>
+    <t xml:space="preserve">$100-200</t>
   </si>
   <si>
     <t xml:space="preserve">Afternoon flight after ferry arrives ~noon</t>
@@ -328,7 +331,7 @@
     <t xml:space="preserve">~1h</t>
   </si>
   <si>
-    <t xml:space="preserve">$50-120</t>
+    <t xml:space="preserve">$75-150</t>
   </si>
   <si>
     <t xml:space="preserve">Short morning hop</t>
@@ -343,22 +346,19 @@
     <t xml:space="preserve">~2.5h</t>
   </si>
   <si>
-    <t xml:space="preserve">$40-100</t>
+    <t xml:space="preserve">$60-140</t>
   </si>
   <si>
     <t xml:space="preserve">Direct to Gatwick, ~2.5h</t>
   </si>
   <si>
-    <t xml:space="preserve">Jun 13</t>
-  </si>
-  <si>
     <t xml:space="preserve">TBD (direct or 1-stop)</t>
   </si>
   <si>
     <t xml:space="preserve">~11h</t>
   </si>
   <si>
-    <t xml:space="preserve">$300-500</t>
+    <t xml:space="preserve">$450-700</t>
   </si>
   <si>
     <t xml:space="preserve">Direct options: BA, Virgin, AA, United, Norse</t>
@@ -367,7 +367,7 @@
     <t xml:space="preserve">LAX &gt; NYC (JFK)</t>
   </si>
   <si>
-    <t xml:space="preserve">Jun 19</t>
+    <t xml:space="preserve">Jun 19 (morning)</t>
   </si>
   <si>
     <t xml:space="preserve">JetBlue / Delta / AA</t>
@@ -376,21 +376,27 @@
     <t xml:space="preserve">~5h</t>
   </si>
   <si>
-    <t xml:space="preserve">$100-250</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Evening departure after dr's appt</t>
+    <t xml:space="preserve">$160-280</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Morning departure, arrive NYC afternoon/evening</t>
   </si>
   <si>
     <t xml:space="preserve">~5.5h</t>
   </si>
   <si>
+    <t xml:space="preserve">$180-350</t>
+  </si>
+  <si>
     <t xml:space="preserve">Person A returns home</t>
   </si>
   <si>
     <t xml:space="preserve">Southwest / AA</t>
   </si>
   <si>
+    <t xml:space="preserve">$170-300</t>
+  </si>
+  <si>
     <t xml:space="preserve">Person B returns after wedding</t>
   </si>
   <si>
@@ -415,7 +421,7 @@
     <t xml:space="preserve">Blue Star / SeaJets / Hellenic</t>
   </si>
   <si>
-    <t xml:space="preserve">$45-80</t>
+    <t xml:space="preserve">$45-85</t>
   </si>
   <si>
     <t xml:space="preserve">Morning departure from Piraeus Gate E7</t>
@@ -427,9 +433,6 @@
     <t xml:space="preserve">May 31 (Sun)</t>
   </si>
   <si>
-    <t xml:space="preserve">$45-70</t>
-  </si>
-  <si>
     <t xml:space="preserve">Early morning departure, arrive Piraeus by noon</t>
   </si>
   <si>
@@ -442,16 +445,16 @@
     <t xml:space="preserve">Est_Cost_Per_Night</t>
   </si>
   <si>
-    <t xml:space="preserve">$120-180</t>
+    <t xml:space="preserve">$160-240</t>
   </si>
   <si>
     <t xml:space="preserve">May 26-27</t>
   </si>
   <si>
-    <t xml:space="preserve">$80-120</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$90-150</t>
+    <t xml:space="preserve">$110-160</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$140-220</t>
   </si>
   <si>
     <t xml:space="preserve">May 29-30</t>
@@ -466,217 +469,226 @@
     <t xml:space="preserve">Zagreb</t>
   </si>
   <si>
+    <t xml:space="preserve">$90-140</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jun 1-2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$140-240</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jun 3-6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Free</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jun 7-13 (free)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$220-380</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jun 19-24 (1 room, 1 bed, 2 ppl)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Category</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Low_Estimate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">High_Estimate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flights (all legs)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$3,680</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$6,230</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9 flights total for 2 ppl + 1 solo BWI&gt;LAX; re-priced for last-minute May 2026 booking</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ferries (Piraeus-Paros RT)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$180</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$340</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 ferries x 2 people</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accommodation (18 paid nights)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$2,880</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$4,760</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 Florence + 1 Athens + 2 Paros + 1 Athens return + 2 Zagreb + 4 Dubrovnik + 0 London (free) + 6 NYC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Food &amp; Drink</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$1,500</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$2,600</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~25 days of eating</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Activities &amp; Entrance Fees</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$400</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$800</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Museums, Plitvice, kayak, cooking class, walls, Kotor bus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Local Transport</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$300</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$500</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buses, metro, taxis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Travel Insurance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$200</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recommended</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL (2 people)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$9,140</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$15,630</t>
+  </si>
+  <si>
+    <t xml:space="preserve">For 2 people total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Food_Per_Day</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transport_Per_Day</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Activities_Per_Day</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$60-90</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$5-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$20-40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Museum passes, gelato budget</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$40-60</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$10-15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$15-25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acropolis ticket ~$22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$50-80</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$10-20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$30-60</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sea kayak ~$105, cooking class ~$123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$0-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Overnight before Zagreb flight</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plitvice day trip base</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plitvice entrance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">day trip</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$30-36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Park entrance ~$25/pp, bus ~$15-18/pp each way</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$15-30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Walls ticket ~$35, Lokrum ferry ~$15, Kotor bus ~$30/pp RT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Free accommodation helps a lot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6</t>
+  </si>
+  <si>
     <t xml:space="preserve">$60-100</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jun 1-2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$80-140</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jun 3-6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Free</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jun 7-13 (free)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$150-250</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jun 18-25 (1 room, 1 bed, 2 ppl)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Category</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Low_Estimate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">High_Estimate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Flights (all legs)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$2,400</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$4,200</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9 flights total for 2 ppl + 1 solo BWI&gt;LAX</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ferries (Piraeus-Paros RT)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$180</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$300</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2 ferries x 2 people</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Accommodation (19 paid nights)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$2,010</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$3,550</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2 Florence + 1 Athens + 2 Paros + 1 Athens return + 2 Zagreb + 4 Dubrovnik + 7 NYC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Food &amp; Drink</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$1,500</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$2,600</t>
-  </si>
-  <si>
-    <t xml:space="preserve">~26 days of eating</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Activities &amp; Entrance Fees</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$400</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$800</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Museums, Plitvice, kayak, cooking class, walls, Kotor bus</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Local Transport</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$500</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Buses, metro, taxis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Travel Insurance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$200</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Recommended</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOTAL (2 people)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$6,990</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$12,350</t>
-  </si>
-  <si>
-    <t xml:space="preserve">For 2 people total</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Food_Per_Day</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Transport_Per_Day</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Activities_Per_Day</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$60-90</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$5-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$20-40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Museum passes, gelato budget</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$40-60</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$10-15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$15-25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Acropolis ticket ~$22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$50-80</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$10-20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$30-60</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sea kayak ~$105, cooking class ~$123</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$0-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Overnight before Zagreb flight</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Plitvice day trip base</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Plitvice entrance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">day trip</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$30-36</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Park entrance ~$25/pp, bus ~$15-18/pp each way</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$15-30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Walls ticket ~$35, Lokrum ferry ~$15, Kotor bus ~$30/pp RT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Free accommodation helps a lot</t>
   </si>
   <si>
     <t xml:space="preserve">1 room 1 bed for 2 ppl</t>
@@ -687,7 +699,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -695,16 +707,27 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <b/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9E1F2"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -712,12 +735,20 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1011,24 +1042,24 @@
     <col min="1" max="1" width="9.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="7.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="23.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="94.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="84.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="16.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1343,7 +1374,7 @@
         <v>69</v>
       </c>
       <c r="B20" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="C20" t="s">
         <v>70</v>
@@ -1369,21 +1400,21 @@
         <v>75</v>
       </c>
       <c r="E21" t="s">
-        <v>61</v>
+        <v>76</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B22" t="s">
         <v>26</v>
       </c>
       <c r="C22" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D22" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E22" t="s">
         <v>9</v>
@@ -1391,16 +1422,16 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B23" t="s">
         <v>30</v>
       </c>
       <c r="C23" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D23" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E23" t="s">
         <v>9</v>
@@ -1418,51 +1449,51 @@
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="29.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="9.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="16.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="38.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="14.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="12.71" hidden="0" customWidth="1"/>
-    <col min="6" max="6" width="72.71" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="70.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s">
-        <v>82</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" t="s">
-        <v>83</v>
-      </c>
-      <c r="D1" t="s">
+      <c r="C1" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="E1" t="s">
+      <c r="D1" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="F1" t="s">
+      <c r="E1" s="1" t="s">
         <v>86</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="F2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="3">
@@ -1473,16 +1504,16 @@
         <v>18</v>
       </c>
       <c r="C3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="4">
@@ -1490,19 +1521,19 @@
         <v>39</v>
       </c>
       <c r="B4" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="D4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E4" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="5">
@@ -1510,39 +1541,39 @@
         <v>45</v>
       </c>
       <c r="B5" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F5" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B6" t="s">
         <v>54</v>
       </c>
       <c r="C6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F6" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="7">
@@ -1550,7 +1581,7 @@
         <v>63</v>
       </c>
       <c r="B7" t="s">
-        <v>110</v>
+        <v>62</v>
       </c>
       <c r="C7" t="s">
         <v>111</v>
@@ -1587,10 +1618,10 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
+        <v>78</v>
+      </c>
+      <c r="B9" t="s">
         <v>77</v>
-      </c>
-      <c r="B9" t="s">
-        <v>76</v>
       </c>
       <c r="C9" t="s">
         <v>117</v>
@@ -1599,30 +1630,30 @@
         <v>121</v>
       </c>
       <c r="E9" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="F9" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
+        <v>81</v>
+      </c>
+      <c r="B10" t="s">
         <v>80</v>
       </c>
-      <c r="B10" t="s">
-        <v>79</v>
-      </c>
       <c r="C10" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D10" t="s">
         <v>121</v>
       </c>
       <c r="E10" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="F10" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
   </sheetData>
@@ -1645,63 +1676,63 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s">
-        <v>125</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" t="s">
-        <v>84</v>
-      </c>
-      <c r="D1" t="s">
-        <v>126</v>
-      </c>
-      <c r="E1" t="s">
-        <v>127</v>
-      </c>
-      <c r="F1" t="s">
-        <v>86</v>
+      <c r="C1" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C2" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D2" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="E2" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="F2" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
+        <v>136</v>
+      </c>
+      <c r="B3" t="s">
+        <v>137</v>
+      </c>
+      <c r="C3" t="s">
+        <v>132</v>
+      </c>
+      <c r="D3" t="s">
+        <v>133</v>
+      </c>
+      <c r="E3" t="s">
         <v>134</v>
       </c>
-      <c r="B3" t="s">
-        <v>135</v>
-      </c>
-      <c r="C3" t="s">
-        <v>130</v>
-      </c>
-      <c r="D3" t="s">
-        <v>131</v>
-      </c>
-      <c r="E3" t="s">
-        <v>136</v>
-      </c>
       <c r="F3" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
   </sheetData>
@@ -1722,17 +1753,17 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s">
-        <v>138</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="D1" t="s">
-        <v>86</v>
+      <c r="C1" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="2">
@@ -1743,10 +1774,10 @@
         <v>2</v>
       </c>
       <c r="C2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="3">
@@ -1757,7 +1788,7 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D3" t="s">
         <v>18</v>
@@ -1771,38 +1802,38 @@
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D4" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B5" t="n">
         <v>1</v>
       </c>
       <c r="C5" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D5" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B6" t="n">
         <v>2</v>
       </c>
       <c r="C6" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D6" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="7">
@@ -1813,10 +1844,10 @@
         <v>4</v>
       </c>
       <c r="C7" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D7" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="8">
@@ -1827,10 +1858,10 @@
         <v>7</v>
       </c>
       <c r="C8" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D8" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="9">
@@ -1838,13 +1869,13 @@
         <v>74</v>
       </c>
       <c r="B9" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C9" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D9" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
   </sheetData>
@@ -1861,133 +1892,133 @@
     <col min="1" max="1" width="30.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="12.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="13.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="82.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="100.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s">
-        <v>157</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="D1" t="s">
-        <v>86</v>
+      <c r="C1" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D2" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B3" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C3" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D3" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B4" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C4" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D4" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B5" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C5" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D5" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B6" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C6" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D6" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B7" t="s">
-        <v>166</v>
+        <v>182</v>
       </c>
       <c r="C7" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="D7" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B8" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C8" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D8" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B9" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="C9" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="D9" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
     </row>
   </sheetData>
@@ -2010,23 +2041,23 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s">
-        <v>138</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="C1" t="s">
-        <v>190</v>
-      </c>
-      <c r="D1" t="s">
-        <v>191</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>192</v>
       </c>
-      <c r="F1" t="s">
-        <v>86</v>
+      <c r="D1" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="2">
@@ -2034,19 +2065,19 @@
         <v>12</v>
       </c>
       <c r="B2" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C2" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="D2" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="E2" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="F2" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
     </row>
     <row r="3">
@@ -2054,19 +2085,19 @@
         <v>23</v>
       </c>
       <c r="B3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C3" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="D3" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="E3" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="F3" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="4">
@@ -2074,79 +2105,79 @@
         <v>27</v>
       </c>
       <c r="B4" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C4" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="D4" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="E4" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="F4" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B5" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C5" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="D5" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="E5" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="F5" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B6" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C6" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="D6" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="E6" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F6" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B7" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="C7" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="D7" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="E7" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="F7" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="8">
@@ -2154,19 +2185,19 @@
         <v>48</v>
       </c>
       <c r="B8" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="C8" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="D8" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="E8" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="F8" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
     </row>
     <row r="9">
@@ -2174,19 +2205,19 @@
         <v>59</v>
       </c>
       <c r="B9" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="C9" t="s">
+        <v>205</v>
+      </c>
+      <c r="D9" t="s">
         <v>203</v>
       </c>
-      <c r="D9" t="s">
-        <v>201</v>
-      </c>
       <c r="E9" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="F9" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
     </row>
     <row r="10">
@@ -2194,19 +2225,19 @@
         <v>74</v>
       </c>
       <c r="B10" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="C10" t="s">
-        <v>149</v>
+        <v>223</v>
       </c>
       <c r="D10" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="E10" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="F10" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
     </row>
   </sheetData>

</xml_diff>